<commit_message>
Correct the national anthem block to the staff line-up
The anthem is a respect moment, not a sales moment. Staff line up behind the
bar facing the projector screen; everything stops — no pouring, running,
ringing or side conversations. Fields are now anthem time and who calls the
floor to stop.

Social media shot list updated to capture the line-up during the anthem.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -706,7 +706,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>NATIONAL ANTHEM — LINE UP</t>
+          <t>NATIONAL ANTHEM</t>
         </is>
       </c>
       <c r="B14" s="7" t="n"/>
@@ -716,38 +716,30 @@
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="7" t="n"/>
     </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Anthem is a moment we own. Shots lined up on the bar BEFORE it starts, not during it. Floor stops, staff stops, nobody runs a plate through it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>When the anthem starts, the staff lines up behind the bar and faces the projector screen. All of you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>ANTHEM TIME:</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>SHOTS LINED UP (WHAT / HOW MANY):</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
+          <t>Everything stops. No pouring, no running food, no ringing tickets, no side conversations. Hands empty, hats off, eyes on the screen. It is ninety seconds, and in a room full of people who have never been here, it is the ninety seconds they remember. Get the floor ready before it starts, not during it.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>WHO IS POURING:</t>
+          <t>ANTHEM TIME:</t>
         </is>
       </c>
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>WHERE THEY LINE UP:</t>
+          <t>WHO CALLS THE FLOOR TO STOP:</t>
         </is>
       </c>
       <c r="F17" s="5" t="n"/>
@@ -1527,7 +1519,7 @@
       </c>
       <c r="B93" s="9" t="inlineStr">
         <is>
-          <t>Anthem time on the board, and the line-up poured before it starts.</t>
+          <t>Anthem time on the board — every staff member knows to line up behind the bar.</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1783,7 @@
       </c>
       <c r="B116" s="9" t="inlineStr">
         <is>
-          <t>Work the room all night, not just the first hour. Get the line-up before the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
+          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
         </is>
       </c>
     </row>
@@ -1960,10 +1952,9 @@
     </row>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="B120:G120"/>
     <mergeCell ref="B117:G117"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="B120:G120"/>
     <mergeCell ref="A108:C108"/>
     <mergeCell ref="B101:G101"/>
     <mergeCell ref="B98:G98"/>
@@ -2006,6 +1997,7 @@
     <mergeCell ref="A33:G34"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="D108:G108"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="B113:G113"/>
     <mergeCell ref="B97:G97"/>
     <mergeCell ref="A90:G90"/>

</xml_diff>

<commit_message>
Move game time and other important notes into the board section
The board now opens with GAME TIME and DOORS and closes with OTHER IMPORTANT
NOTES, so everything a manager writes on the board is in one block instead of
split between the header and the bottom of the sheet.

Header keeps date, day, shift, matchup, expected volume and manager on duty.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Game Day Pre-Shift" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$136</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.5" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,7 @@
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>KICKOFF:</t>
+          <t>EXPECTED VOLUME:</t>
         </is>
       </c>
       <c r="F5" s="5" t="n"/>
@@ -629,139 +629,136 @@
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>DOORS:</t>
+          <t>MANAGER ON DUTY:</t>
         </is>
       </c>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>MANAGER ON DUTY:</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>EXPECTED VOLUME:</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>THE THREE WINDOWS — WRITE THE TIMES ON THE BOARD</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>PRE-GAME</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Volume and speed, turn-and-burn. Guests have a hard out.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>PRE-GAME</t>
+          <t>GAME WINDOW</t>
         </is>
       </c>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Volume and speed, turn-and-burn. Guests have a hard out.</t>
+          <t>Floor thins, bar fills. It feels slow. It is not — it is the setup.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>GAME WINDOW</t>
+          <t>POST-GAME</t>
         </is>
       </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Floor thins, bar fills. It feels slow. It is not — it is the setup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>POST-GAME</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
           <t>Hardest 90 minutes of the week. All hands on the floor before the final whistle.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>NATIONAL ANTHEM</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>When the anthem starts, the staff lines up behind the bar and faces the projector screen. All of you.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="44" customHeight="1">
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Everything stops. No pouring, no running food, no ringing tickets, no side conversations. Hands empty, hats off, eyes on the screen. It is ninety seconds, and in a room full of people who have never been here, it is the ninety seconds they remember. Get the floor ready before it starts, not during it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Everything stops. No pouring, no running food, no ringing tickets, no side conversations. Hands empty, hats off, eyes on the screen. It is ninety seconds, and in a room full of people who have never been here, it is the ninety seconds they remember. Get the floor ready before it starts, not during it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
           <t>ANTHEM TIME:</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>WHO CALLS THE FLOOR TO STOP:</t>
         </is>
       </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>THE THREE HARD LINES — SAY ALL THREE OUT LOUD, EVERY GAME DAY</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>1.  NO DRINKING — not before your shift, not on your shift, not on the clock in any capacity. Not a taste, not a guest-bought round, not overtime.</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>1.  NO DRINKING — not before your shift, not on your shift, not on the clock in any capacity. Not a taste, not a guest-bought round, not overtime.</t>
+          <t>2.  NO PROMO BOTTLES — no bottle leaves the bar as a promo, comp, gift or bucket. Every bottle rings in and gets paid for. Every single one.</t>
         </is>
       </c>
       <c r="B20" s="13" t="n"/>
@@ -774,7 +771,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2.  NO PROMO BOTTLES — no bottle leaves the bar as a promo, comp, gift or bucket. Every bottle rings in and gets paid for. Every single one.</t>
+          <t>3.  NO DISCOUNTS — every check rings at full price. No employee rate for a friend, no "take care of them." You do not have discount authority.</t>
         </is>
       </c>
       <c r="B21" s="13" t="n"/>
@@ -785,9 +782,9 @@
       <c r="G21" s="13" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>3.  NO DISCOUNTS — every check rings at full price. No employee rate for a friend, no "take care of them." You do not have discount authority.</t>
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>NOTE: a promo bottle is NOT bottle service. Bottle service is a product we SELL and ring at full price — sell it hard. A promo bottle is one that leaves with no ticket. Sell every bottle. Give away none.</t>
         </is>
       </c>
       <c r="B22" s="13" t="n"/>
@@ -800,7 +797,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>NOTE: a promo bottle is NOT bottle service. Bottle service is a product we SELL and ring at full price — sell it hard. A promo bottle is one that leaves with no ticket. Sell every bottle. Give away none.</t>
+          <t>If a guest needs to be taken care of, GET A MANAGER. You will never get in trouble for getting a manager. You will get in trouble for making the call yourself.</t>
         </is>
       </c>
       <c r="B23" s="13" t="n"/>
@@ -810,36 +807,36 @@
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="13" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>If a guest needs to be taken care of, GET A MANAGER. You will never get in trouble for getting a manager. You will get in trouble for making the call yourself.</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>ID'ING — NO EXCEPTIONS, NOT ON GAME DAY</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="11" t="n"/>
-      <c r="F26" s="11" t="n"/>
-      <c r="G26" s="11" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Every guest who looks under 40 gets carded. Every time. At the bar, at the table, and again if someone hands them a drink they did not order.</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Every guest who looks under 40 gets carded. Every time. At the bar, at the table, and again if someone hands them a drink they did not order.</t>
+          <t>Physical ID only. Expired is not an ID. A vertical license means look twice and do the math out loud.</t>
         </is>
       </c>
       <c r="B27" s="13" t="n"/>
@@ -852,7 +849,7 @@
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Physical ID only. Expired is not an ID. A vertical license means look twice and do the math out loud.</t>
+          <t>If you are not sure, you do not pour. Hand it to a manager — that is the whole process, and nobody gets second-guessed for using it.</t>
         </is>
       </c>
       <c r="B28" s="13" t="n"/>
@@ -865,7 +862,7 @@
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>If you are not sure, you do not pour. Hand it to a manager — that is the whole process, and nobody gets second-guessed for using it.</t>
+          <t>Game day is the night we get tested on this. The liquor license is the entire business. One bad pour costs more than the whole night made.</t>
         </is>
       </c>
       <c r="B29" s="13" t="n"/>
@@ -875,520 +872,478 @@
       <c r="F29" s="13" t="n"/>
       <c r="G29" s="13" t="n"/>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>Game day is the night we get tested on this. The liquor license is the entire business. One bad pour costs more than the whole night made.</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="n"/>
-      <c r="C30" s="13" t="n"/>
-      <c r="D30" s="13" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
-      <c r="G30" s="13" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>THE BOARD</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+    </row>
+    <row r="32" ht="19" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>GAME TIME:</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>DOORS:</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>GOAL / CONTEST FOR THE DAY:</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="16" t="n"/>
-      <c r="B33" s="17" t="n"/>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="17" t="n"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="17" t="n"/>
-      <c r="B34" s="17" t="n"/>
-      <c r="C34" s="17" t="n"/>
-      <c r="D34" s="17" t="n"/>
-      <c r="E34" s="17" t="n"/>
-      <c r="F34" s="17" t="n"/>
-      <c r="G34" s="17" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="16" t="n"/>
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="17" t="n"/>
+      <c r="D35" s="17" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17" t="n"/>
+      <c r="G35" s="17" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="17" t="n"/>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="17" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="17" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>NEW BEERS / NEW ITEMS:</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="16" t="n"/>
-      <c r="B37" s="17" t="n"/>
-      <c r="C37" s="17" t="n"/>
-      <c r="D37" s="17" t="n"/>
-      <c r="E37" s="17" t="n"/>
-      <c r="F37" s="17" t="n"/>
-      <c r="G37" s="17" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="17" t="n"/>
-      <c r="B38" s="17" t="n"/>
-      <c r="C38" s="17" t="n"/>
-      <c r="D38" s="17" t="n"/>
-      <c r="E38" s="17" t="n"/>
-      <c r="F38" s="17" t="n"/>
-      <c r="G38" s="17" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="16" t="n"/>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="17" t="n"/>
+      <c r="D39" s="17" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="17" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="17" t="n"/>
+      <c r="D40" s="17" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="17" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>86:</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="16" t="n"/>
-      <c r="B41" s="17" t="n"/>
-      <c r="C41" s="17" t="n"/>
-      <c r="D41" s="17" t="n"/>
-      <c r="E41" s="17" t="n"/>
-      <c r="F41" s="17" t="n"/>
-      <c r="G41" s="17" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="17" t="n"/>
-      <c r="B42" s="17" t="n"/>
-      <c r="C42" s="17" t="n"/>
-      <c r="D42" s="17" t="n"/>
-      <c r="E42" s="17" t="n"/>
-      <c r="F42" s="17" t="n"/>
-      <c r="G42" s="17" t="n"/>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="16" t="n"/>
+      <c r="B43" s="17" t="n"/>
+      <c r="C43" s="17" t="n"/>
+      <c r="D43" s="17" t="n"/>
+      <c r="E43" s="17" t="n"/>
+      <c r="F43" s="17" t="n"/>
+      <c r="G43" s="17" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="17" t="n"/>
+      <c r="B44" s="17" t="n"/>
+      <c r="C44" s="17" t="n"/>
+      <c r="D44" s="17" t="n"/>
+      <c r="E44" s="17" t="n"/>
+      <c r="F44" s="17" t="n"/>
+      <c r="G44" s="17" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>OTHER IMPORTANT NOTES:</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="16" t="n"/>
+      <c r="B47" s="17" t="n"/>
+      <c r="C47" s="17" t="n"/>
+      <c r="D47" s="17" t="n"/>
+      <c r="E47" s="17" t="n"/>
+      <c r="F47" s="17" t="n"/>
+      <c r="G47" s="17" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="17" t="n"/>
+      <c r="B48" s="17" t="n"/>
+      <c r="C48" s="17" t="n"/>
+      <c r="D48" s="17" t="n"/>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="17" t="n"/>
+      <c r="G48" s="17" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>PROMOS FOR THE DAY — EVERYBODY KNOWS ALL THREE BEFORE DOORS</t>
         </is>
       </c>
-      <c r="B44" s="7" t="n"/>
-      <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
-      <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="n"/>
-      <c r="G44" s="7" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>Suncruiser Buckets</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C51" s="18" t="inlineStr">
         <is>
           <t>6 / 30</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="D51" s="9" t="inlineStr">
         <is>
           <t>Lead with this at every table in the pre-game window. Fastest ticket in the building.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Lucky One Lemonade</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C52" s="18" t="inlineStr">
         <is>
           <t>6 / 24</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="D52" s="9" t="inlineStr">
         <is>
           <t>Same play. Buckets land on the table before the first food order goes in.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
         <is>
           <t>Tito's Bottle Service</t>
         </is>
       </c>
-      <c r="C47" s="19" t="inlineStr">
+      <c r="C53" s="19" t="inlineStr">
         <is>
           <t>PUSH HARD</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D53" s="9" t="inlineStr">
         <is>
           <t>The one we are chasing tonight. Offer it to every large party, every booth, every group already celebrating. Rings at full price — bottle service is sold, never comped.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="9" t="inlineStr">
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>Other promos:</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="5" t="n"/>
-      <c r="G48" s="5" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="5" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>STAFF #'S</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>SHIFT LEADS:</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>STAFF TO COACH:</t>
         </is>
       </c>
-    </row>
-    <row r="51" ht="19" customHeight="1">
-      <c r="A51" s="20" t="inlineStr">
-        <is>
-          <t>SERVERS:</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>1 HUDDL COMPLETION</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="19" customHeight="1">
-      <c r="A52" s="20" t="inlineStr">
-        <is>
-          <t>BARTENDERS:</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="n"/>
-    </row>
-    <row r="53" ht="19" customHeight="1">
-      <c r="A53" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n"/>
-      <c r="C53" s="20" t="inlineStr">
-        <is>
-          <t>BARTENDER:</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="n"/>
-    </row>
-    <row r="54" ht="19" customHeight="1">
-      <c r="A54" s="20" t="inlineStr">
-        <is>
-          <t>HOSTS:</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n"/>
-      <c r="C54" s="20" t="inlineStr">
-        <is>
-          <t>HOST:</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="n"/>
-    </row>
-    <row r="55" ht="19" customHeight="1">
-      <c r="A55" s="20" t="inlineStr">
-        <is>
-          <t>RUNNERS:</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="n"/>
-      <c r="C55" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="20" t="inlineStr">
-        <is>
-          <t>HOST:</t>
-        </is>
-      </c>
-      <c r="F55" s="5" t="n"/>
-    </row>
-    <row r="56" ht="19" customHeight="1">
-      <c r="A56" s="20" t="inlineStr">
-        <is>
-          <t>BARBACKS:</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="20" t="inlineStr">
-        <is>
-          <t>BARBACK:</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="20" t="inlineStr">
-        <is>
-          <t>BARBACK:</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="n"/>
     </row>
     <row r="57" ht="19" customHeight="1">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>SHOT GIRL:</t>
+          <t>SERVERS:</t>
         </is>
       </c>
       <c r="B57" s="5" t="n"/>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>1 HUDDL COMPLETION</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="19" customHeight="1">
       <c r="A58" s="20" t="inlineStr">
         <is>
+          <t>BARTENDERS:</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n"/>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="n"/>
+    </row>
+    <row r="59" ht="19" customHeight="1">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n"/>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>BARTENDER:</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="n"/>
+    </row>
+    <row r="60" ht="19" customHeight="1">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>HOSTS:</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n"/>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="n"/>
+    </row>
+    <row r="61" ht="19" customHeight="1">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>RUNNERS:</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="n"/>
+    </row>
+    <row r="62" ht="19" customHeight="1">
+      <c r="A62" s="20" t="inlineStr">
+        <is>
+          <t>BARBACKS:</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="n"/>
+    </row>
+    <row r="63" ht="19" customHeight="1">
+      <c r="A63" s="20" t="inlineStr">
+        <is>
+          <t>SHOT GIRL:</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n"/>
+    </row>
+    <row r="64" ht="19" customHeight="1">
+      <c r="A64" s="20" t="inlineStr">
+        <is>
           <t>MANAGERS:</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n"/>
-    </row>
-    <row r="60">
-      <c r="E60" s="4" t="inlineStr">
+      <c r="B64" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>7SHIFTS COMPLETION</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="E61" s="20" t="inlineStr">
+    <row r="67">
+      <c r="E67" s="20" t="inlineStr">
         <is>
           <t>SERVER:</t>
         </is>
       </c>
-      <c r="F61" s="5" t="n"/>
-    </row>
-    <row r="62">
-      <c r="E62" s="20" t="inlineStr">
+      <c r="F67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="E68" s="20" t="inlineStr">
         <is>
           <t>BAR:</t>
         </is>
       </c>
-      <c r="F62" s="5" t="n"/>
-    </row>
-    <row r="63">
-      <c r="E63" s="20" t="inlineStr">
+      <c r="F68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="E69" s="20" t="inlineStr">
         <is>
           <t>CAFÉ:</t>
         </is>
       </c>
-      <c r="F63" s="5" t="n"/>
-    </row>
-    <row r="64">
-      <c r="E64" s="20" t="inlineStr">
+      <c r="F69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="E70" s="20" t="inlineStr">
         <is>
           <t>HOST:</t>
         </is>
       </c>
-      <c r="F64" s="5" t="n"/>
-    </row>
-    <row r="65">
-      <c r="E65" s="20" t="inlineStr">
+      <c r="F70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="E71" s="20" t="inlineStr">
         <is>
           <t>BARBACK:</t>
         </is>
       </c>
-      <c r="F65" s="5" t="n"/>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="6" t="inlineStr">
+      <c r="F71" s="5" t="n"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
         <is>
           <t>STATION ASSIGNMENTS — WRITE A NAME ON EVERY LINE</t>
         </is>
       </c>
-      <c r="B67" s="7" t="n"/>
-      <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="n"/>
-      <c r="E67" s="7" t="n"/>
-      <c r="F67" s="7" t="n"/>
-      <c r="G67" s="7" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="B73" s="7" t="n"/>
+      <c r="C73" s="7" t="n"/>
+      <c r="D73" s="7" t="n"/>
+      <c r="E73" s="7" t="n"/>
+      <c r="F73" s="7" t="n"/>
+      <c r="G73" s="7" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>HOST</t>
         </is>
       </c>
-      <c r="C68" s="8" t="inlineStr">
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>RUNNERS</t>
         </is>
       </c>
-      <c r="E68" s="8" t="inlineStr">
+      <c r="E74" s="8" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="9" t="inlineStr">
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>Lead:</t>
         </is>
       </c>
-      <c r="B69" s="5" t="n"/>
-      <c r="C69" s="9" t="inlineStr">
+      <c r="B75" s="5" t="n"/>
+      <c r="C75" s="9" t="inlineStr">
         <is>
           <t>Bar 100:</t>
         </is>
       </c>
-      <c r="D69" s="5" t="n"/>
-      <c r="E69" s="9" t="inlineStr">
+      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="9" t="inlineStr">
         <is>
           <t>100:</t>
         </is>
       </c>
-      <c r="F69" s="5" t="n"/>
-      <c r="G69" s="5" t="n"/>
-    </row>
-    <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="9" t="inlineStr">
-        <is>
-          <t>Runner:</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="n"/>
-      <c r="C70" s="9" t="inlineStr">
-        <is>
-          <t>Bar 200:</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="n"/>
-      <c r="E70" s="9" t="inlineStr">
-        <is>
-          <t>105:</t>
-        </is>
-      </c>
-      <c r="F70" s="5" t="n"/>
-      <c r="G70" s="5" t="n"/>
-    </row>
-    <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="9" t="inlineStr">
-        <is>
-          <t>Waters:</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="n"/>
-      <c r="C71" s="9" t="inlineStr">
-        <is>
-          <t>Food:</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="n"/>
-      <c r="E71" s="9" t="inlineStr">
-        <is>
-          <t>110:</t>
-        </is>
-      </c>
-      <c r="F71" s="5" t="n"/>
-      <c r="G71" s="5" t="n"/>
-    </row>
-    <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="9" t="inlineStr">
-        <is>
-          <t>Bathrooms:</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="n"/>
-      <c r="E72" s="9" t="inlineStr">
-        <is>
-          <t>200:</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="n"/>
-      <c r="G72" s="5" t="n"/>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>Patio:</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="n"/>
-      <c r="G73" s="5" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
-        <is>
-          <t>BARBACKS</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>SHOT GIRL</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>TASTE PLATE</t>
-        </is>
-      </c>
+      <c r="F75" s="5" t="n"/>
+      <c r="G75" s="5" t="n"/>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>Main Bar:</t>
+          <t>Runner:</t>
         </is>
       </c>
       <c r="B76" s="5" t="n"/>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>On tonight:</t>
+          <t>Bar 200:</t>
         </is>
       </c>
       <c r="D76" s="5" t="n"/>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Running it:</t>
+          <t>105:</t>
         </is>
       </c>
       <c r="F76" s="5" t="n"/>
@@ -1397,46 +1352,90 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>Patio Bar:</t>
+          <t>Waters:</t>
         </is>
       </c>
       <c r="B77" s="5" t="n"/>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>Food:</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="n"/>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>110:</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="n"/>
+      <c r="G77" s="5" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Main Floor:</t>
+          <t>Bathrooms:</t>
         </is>
       </c>
       <c r="B78" s="5" t="n"/>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>200:</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="n"/>
+      <c r="G78" s="5" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="9" t="inlineStr">
-        <is>
-          <t>Café:</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="n"/>
-    </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="9" t="inlineStr">
-        <is>
-          <t>Front Patio:</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t>SOCIAL MEDIA</t>
-        </is>
-      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>Patio:</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="n"/>
+      <c r="G79" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>BARBACKS</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>SHOT GIRL</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>TASTE PLATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>Main Bar:</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>Running it:</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="n"/>
+      <c r="G82" s="5" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>On tonight:</t>
+          <t>Patio Bar:</t>
         </is>
       </c>
       <c r="B83" s="5" t="n"/>
@@ -1444,120 +1443,87 @@
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
         <is>
+          <t>Main Floor:</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n"/>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>Café:</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="n"/>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>Front Patio:</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL MEDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B84" s="5" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
+      <c r="B90" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>PARTIES / EVENTS:</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="16" t="n"/>
-      <c r="B87" s="17" t="n"/>
-      <c r="C87" s="17" t="n"/>
-      <c r="D87" s="17" t="n"/>
-      <c r="E87" s="17" t="n"/>
-      <c r="F87" s="17" t="n"/>
-      <c r="G87" s="17" t="n"/>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="17" t="n"/>
-      <c r="B88" s="17" t="n"/>
-      <c r="C88" s="17" t="n"/>
-      <c r="D88" s="17" t="n"/>
-      <c r="E88" s="17" t="n"/>
-      <c r="F88" s="17" t="n"/>
-      <c r="G88" s="17" t="n"/>
-    </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="6" t="inlineStr">
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="16" t="n"/>
+      <c r="B93" s="17" t="n"/>
+      <c r="C93" s="17" t="n"/>
+      <c r="D93" s="17" t="n"/>
+      <c r="E93" s="17" t="n"/>
+      <c r="F93" s="17" t="n"/>
+      <c r="G93" s="17" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="17" t="n"/>
+      <c r="B94" s="17" t="n"/>
+      <c r="C94" s="17" t="n"/>
+      <c r="D94" s="17" t="n"/>
+      <c r="E94" s="17" t="n"/>
+      <c r="F94" s="17" t="n"/>
+      <c r="G94" s="17" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>GAME DAY OPEN — 90 MINUTES BEFORE DOORS</t>
         </is>
       </c>
-      <c r="B90" s="7" t="n"/>
-      <c r="C90" s="7" t="n"/>
-      <c r="D90" s="7" t="n"/>
-      <c r="E90" s="7" t="n"/>
-      <c r="F90" s="7" t="n"/>
-      <c r="G90" s="7" t="n"/>
-    </row>
-    <row r="91" ht="17" customHeight="1">
-      <c r="A91" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B91" s="9" t="inlineStr">
-        <is>
-          <t>Know the game — kickoff, attendance, national TV, weather. Times on the board.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="17" customHeight="1">
-      <c r="A92" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B92" s="9" t="inlineStr">
-        <is>
-          <t>Every staff member can name all three promos — ask two people at random before pre-shift ends.</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="17" customHeight="1">
-      <c r="A93" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B93" s="9" t="inlineStr">
-        <is>
-          <t>Anthem time on the board — every staff member knows to line up behind the bar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="17" customHeight="1">
-      <c r="A94" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B94" s="9" t="inlineStr">
-        <is>
-          <t>Social media assigned, phone charged, and they know the shot list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="17" customHeight="1">
-      <c r="A95" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B95" s="9" t="inlineStr">
-        <is>
-          <t>Three windows built on paper — cut times, breaks, post-game all-hands decided now.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="17" customHeight="1">
-      <c r="A96" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B96" s="9" t="inlineStr">
-        <is>
-          <t>Staffing confirmed against 7shifts. One no-show on game day is a two-hour wait.</t>
-        </is>
-      </c>
+      <c r="B96" s="7" t="n"/>
+      <c r="C96" s="7" t="n"/>
+      <c r="D96" s="7" t="n"/>
+      <c r="E96" s="7" t="n"/>
+      <c r="F96" s="7" t="n"/>
+      <c r="G96" s="7" t="n"/>
     </row>
     <row r="97" ht="17" customHeight="1">
       <c r="A97" s="21" t="inlineStr">
@@ -1567,7 +1533,7 @@
       </c>
       <c r="B97" s="9" t="inlineStr">
         <is>
-          <t>Every station walked, front and back. The 3 Rules on all of them.</t>
+          <t>Know the game — kickoff, attendance, national TV, weather. Times on the board.</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1545,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>Bar par DOUBLED — ice, kegs, backups, garnish, glassware, batch.</t>
+          <t>Every staff member can name all three promos — ask two people at random before pre-shift ends.</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1557,7 @@
       </c>
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>86 board walked with the kitchen, current and visible.</t>
+          <t>Anthem time on the board — every staff member knows to line up behind the bar.</t>
         </is>
       </c>
     </row>
@@ -1603,7 +1569,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>TVs, sound and the game feed tested before a single guest sits down.</t>
+          <t>Social media assigned, phone charged, and they know the shot list.</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1581,7 @@
       </c>
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>ID check covered — door and bar know who is carding, and the light works.</t>
+          <t>Three windows built on paper — cut times, breaks, post-game all-hands decided now.</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1593,7 @@
       </c>
       <c r="B102" s="9" t="inlineStr">
         <is>
-          <t>Restrooms stocked and clean before doors.</t>
+          <t>Staffing confirmed against 7shifts. One no-show on game day is a two-hour wait.</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1605,7 @@
       </c>
       <c r="B103" s="9" t="inlineStr">
         <is>
-          <t>POS, printers and card processing tested with a live ticket.</t>
+          <t>Every station walked, front and back. The 3 Rules on all of them.</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1617,7 @@
       </c>
       <c r="B104" s="9" t="inlineStr">
         <is>
-          <t>Cash on hand for a bar that will run cash all night.</t>
+          <t>Bar par DOUBLED — ice, kegs, backups, garnish, glassware, batch.</t>
         </is>
       </c>
     </row>
@@ -1663,279 +1629,308 @@
       </c>
       <c r="B105" s="9" t="inlineStr">
         <is>
+          <t>86 board walked with the kitchen, current and visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="17" customHeight="1">
+      <c r="A106" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>TVs, sound and the game feed tested before a single guest sits down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="17" customHeight="1">
+      <c r="A107" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>ID check covered — door and bar know who is carding, and the light works.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="17" customHeight="1">
+      <c r="A108" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>Restrooms stocked and clean before doors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="17" customHeight="1">
+      <c r="A109" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>POS, printers and card processing tested with a live ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="17" customHeight="1">
+      <c r="A110" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>Cash on hand for a bar that will run cash all night.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="17" customHeight="1">
+      <c r="A111" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B111" s="9" t="inlineStr">
+        <is>
           <t>Door, patio and line plan — where the wait forms and who holds it.</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="20" customHeight="1">
-      <c r="A107" s="22" t="inlineStr">
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="22" t="inlineStr">
         <is>
           <t>IS STAFF IN UNIFORM?   YES / NO</t>
         </is>
       </c>
-      <c r="B107" s="13" t="n"/>
-      <c r="C107" s="13" t="n"/>
-      <c r="D107" s="22" t="inlineStr">
+      <c r="B113" s="13" t="n"/>
+      <c r="C113" s="13" t="n"/>
+      <c r="D113" s="22" t="inlineStr">
         <is>
           <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
         </is>
       </c>
-      <c r="E107" s="13" t="n"/>
-      <c r="F107" s="13" t="n"/>
-      <c r="G107" s="13" t="n"/>
-    </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="A108" s="22" t="inlineStr">
+      <c r="E113" s="13" t="n"/>
+      <c r="F113" s="13" t="n"/>
+      <c r="G113" s="13" t="n"/>
+    </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="22" t="inlineStr">
         <is>
           <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
         </is>
       </c>
-      <c r="B108" s="13" t="n"/>
-      <c r="C108" s="13" t="n"/>
-      <c r="D108" s="22" t="inlineStr">
+      <c r="B114" s="13" t="n"/>
+      <c r="C114" s="13" t="n"/>
+      <c r="D114" s="22" t="inlineStr">
         <is>
           <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
         </is>
       </c>
-      <c r="E108" s="13" t="n"/>
-      <c r="F108" s="13" t="n"/>
-      <c r="G108" s="13" t="n"/>
-    </row>
-    <row r="109" ht="20" customHeight="1">
-      <c r="A109" s="22" t="inlineStr">
+      <c r="E114" s="13" t="n"/>
+      <c r="F114" s="13" t="n"/>
+      <c r="G114" s="13" t="n"/>
+    </row>
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="22" t="inlineStr">
         <is>
           <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
         </is>
       </c>
-      <c r="B109" s="13" t="n"/>
-      <c r="C109" s="13" t="n"/>
-      <c r="D109" s="13" t="n"/>
-      <c r="E109" s="13" t="n"/>
-      <c r="F109" s="13" t="n"/>
-      <c r="G109" s="13" t="n"/>
-    </row>
-    <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="6" t="inlineStr">
+      <c r="B115" s="13" t="n"/>
+      <c r="C115" s="13" t="n"/>
+      <c r="D115" s="13" t="n"/>
+      <c r="E115" s="13" t="n"/>
+      <c r="F115" s="13" t="n"/>
+      <c r="G115" s="13" t="n"/>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
         </is>
       </c>
-      <c r="B111" s="7" t="n"/>
-      <c r="C111" s="7" t="n"/>
-      <c r="D111" s="7" t="n"/>
-      <c r="E111" s="7" t="n"/>
-      <c r="F111" s="7" t="n"/>
-      <c r="G111" s="7" t="n"/>
-    </row>
-    <row r="112" ht="32" customHeight="1">
-      <c r="A112" s="8" t="inlineStr">
+      <c r="B117" s="7" t="n"/>
+      <c r="C117" s="7" t="n"/>
+      <c r="D117" s="7" t="n"/>
+      <c r="E117" s="7" t="n"/>
+      <c r="F117" s="7" t="n"/>
+      <c r="G117" s="7" t="n"/>
+    </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="A118" s="8" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
-      <c r="B112" s="9" t="inlineStr">
+      <c r="B118" s="9" t="inlineStr">
         <is>
           <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="32" customHeight="1">
-      <c r="A113" s="8" t="inlineStr">
+    <row r="119" ht="32" customHeight="1">
+      <c r="A119" s="8" t="inlineStr">
         <is>
           <t>SERVERS</t>
         </is>
       </c>
-      <c r="B113" s="9" t="inlineStr">
+      <c r="B119" s="9" t="inlineStr">
         <is>
           <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="32" customHeight="1">
-      <c r="A114" s="8" t="inlineStr">
+    <row r="120" ht="32" customHeight="1">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t>HOST</t>
         </is>
       </c>
-      <c r="B114" s="9" t="inlineStr">
+      <c r="B120" s="9" t="inlineStr">
         <is>
           <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. Card at the door when the room is young; it is far easier there than at the bar. Keep the line off the sidewalk and feed the wait to the bar.</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="32" customHeight="1">
-      <c r="A115" s="8" t="inlineStr">
+    <row r="121" ht="32" customHeight="1">
+      <c r="A121" s="8" t="inlineStr">
         <is>
           <t>KITCHEN</t>
         </is>
       </c>
-      <c r="B115" s="9" t="inlineStr">
+      <c r="B121" s="9" t="inlineStr">
         <is>
           <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="32" customHeight="1">
-      <c r="A116" s="8" t="inlineStr">
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="8" t="inlineStr">
         <is>
           <t>SOCIAL</t>
         </is>
       </c>
-      <c r="B116" s="9" t="inlineStr">
+      <c r="B122" s="9" t="inlineStr">
         <is>
           <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="32" customHeight="1">
-      <c r="A117" s="8" t="inlineStr">
+    <row r="123" ht="32" customHeight="1">
+      <c r="A123" s="8" t="inlineStr">
         <is>
           <t>SUPPORT</t>
         </is>
       </c>
-      <c r="B117" s="9" t="inlineStr">
+      <c r="B123" s="9" t="inlineStr">
         <is>
           <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="6" t="inlineStr">
+    <row r="125" ht="18" customHeight="1">
+      <c r="A125" s="6" t="inlineStr">
         <is>
           <t>POST-GAME &amp; CLOSE</t>
         </is>
       </c>
-      <c r="B119" s="7" t="n"/>
-      <c r="C119" s="7" t="n"/>
-      <c r="D119" s="7" t="n"/>
-      <c r="E119" s="7" t="n"/>
-      <c r="F119" s="7" t="n"/>
-      <c r="G119" s="7" t="n"/>
-    </row>
-    <row r="120" ht="17" customHeight="1">
-      <c r="A120" s="21" t="inlineStr">
+      <c r="B125" s="7" t="n"/>
+      <c r="C125" s="7" t="n"/>
+      <c r="D125" s="7" t="n"/>
+      <c r="E125" s="7" t="n"/>
+      <c r="F125" s="7" t="n"/>
+      <c r="G125" s="7" t="n"/>
+    </row>
+    <row r="126" ht="17" customHeight="1">
+      <c r="A126" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B120" s="9" t="inlineStr">
+      <c r="B126" s="9" t="inlineStr">
         <is>
           <t>All hands on the floor BEFORE the final whistle — not after.</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="17" customHeight="1">
-      <c r="A121" s="21" t="inlineStr">
+    <row r="127" ht="17" customHeight="1">
+      <c r="A127" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B121" s="9" t="inlineStr">
+      <c r="B127" s="9" t="inlineStr">
         <is>
           <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="17" customHeight="1">
-      <c r="A122" s="21" t="inlineStr">
+    <row r="128" ht="17" customHeight="1">
+      <c r="A128" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B122" s="9" t="inlineStr">
+      <c r="B128" s="9" t="inlineStr">
         <is>
           <t>Every void, comp and discount reconciled to a manager name.</t>
         </is>
       </c>
     </row>
-    <row r="123" ht="17" customHeight="1">
-      <c r="A123" s="21" t="inlineStr">
+    <row r="129" ht="17" customHeight="1">
+      <c r="A129" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B123" s="9" t="inlineStr">
+      <c r="B129" s="9" t="inlineStr">
         <is>
           <t>Every refusal or cut-off logged with what happened and who made the call.</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="17" customHeight="1">
-      <c r="A124" s="21" t="inlineStr">
+    <row r="130" ht="17" customHeight="1">
+      <c r="A130" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B124" s="9" t="inlineStr">
+      <c r="B130" s="9" t="inlineStr">
         <is>
           <t>Every station back to original position, original condition.</t>
         </is>
       </c>
     </row>
-    <row r="125" ht="17" customHeight="1">
-      <c r="A125" s="21" t="inlineStr">
+    <row r="131" ht="17" customHeight="1">
+      <c r="A131" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B125" s="9" t="inlineStr">
+      <c r="B131" s="9" t="inlineStr">
         <is>
           <t>Shift notes written: what we ran out of, where the wait broke down, what changes next game.</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="4" t="inlineStr">
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
         <is>
           <t>MARKETING:</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="18" customHeight="1">
-      <c r="A128" s="16" t="n"/>
-      <c r="B128" s="17" t="n"/>
-      <c r="C128" s="17" t="n"/>
-      <c r="D128" s="17" t="n"/>
-      <c r="E128" s="17" t="n"/>
-      <c r="F128" s="17" t="n"/>
-      <c r="G128" s="17" t="n"/>
-    </row>
-    <row r="129" ht="18" customHeight="1">
-      <c r="A129" s="17" t="n"/>
-      <c r="B129" s="17" t="n"/>
-      <c r="C129" s="17" t="n"/>
-      <c r="D129" s="17" t="n"/>
-      <c r="E129" s="17" t="n"/>
-      <c r="F129" s="17" t="n"/>
-      <c r="G129" s="17" t="n"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="4" t="inlineStr">
-        <is>
-          <t>OTHER IMPORTANT NOTES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="18" customHeight="1">
-      <c r="A132" s="16" t="n"/>
-      <c r="B132" s="17" t="n"/>
-      <c r="C132" s="17" t="n"/>
-      <c r="D132" s="17" t="n"/>
-      <c r="E132" s="17" t="n"/>
-      <c r="F132" s="17" t="n"/>
-      <c r="G132" s="17" t="n"/>
-    </row>
-    <row r="133" ht="18" customHeight="1">
-      <c r="A133" s="17" t="n"/>
-      <c r="B133" s="17" t="n"/>
-      <c r="C133" s="17" t="n"/>
-      <c r="D133" s="17" t="n"/>
-      <c r="E133" s="17" t="n"/>
-      <c r="F133" s="17" t="n"/>
-      <c r="G133" s="17" t="n"/>
-    </row>
     <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="17" t="n"/>
+      <c r="A134" s="16" t="n"/>
       <c r="B134" s="17" t="n"/>
       <c r="C134" s="17" t="n"/>
       <c r="D134" s="17" t="n"/>
@@ -1943,82 +1938,92 @@
       <c r="F134" s="17" t="n"/>
       <c r="G134" s="17" t="n"/>
     </row>
-    <row r="136" ht="28" customHeight="1">
-      <c r="A136" s="23" t="inlineStr">
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="17" t="n"/>
+      <c r="C135" s="17" t="n"/>
+      <c r="D135" s="17" t="n"/>
+      <c r="E135" s="17" t="n"/>
+      <c r="F135" s="17" t="n"/>
+      <c r="G135" s="17" t="n"/>
+    </row>
+    <row r="137" ht="28" customHeight="1">
+      <c r="A137" s="23" t="inlineStr">
         <is>
           <t>100% of our standards, 100% of the time, at 100% volume. A full house is not an excuse to run at 80% — it is the reason we hold the line.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="68">
+  <mergeCells count="69">
+    <mergeCell ref="C16:E16"/>
     <mergeCell ref="B120:G120"/>
-    <mergeCell ref="B117:G117"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A108:C108"/>
+    <mergeCell ref="B111:G111"/>
+    <mergeCell ref="B107:G107"/>
     <mergeCell ref="B101:G101"/>
+    <mergeCell ref="A8:G8"/>
     <mergeCell ref="B98:G98"/>
-    <mergeCell ref="A128:G129"/>
+    <mergeCell ref="D114:G114"/>
     <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A109:G109"/>
     <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A96:G96"/>
+    <mergeCell ref="A125:G125"/>
     <mergeCell ref="A29:G29"/>
+    <mergeCell ref="B119:G119"/>
+    <mergeCell ref="D51:G51"/>
     <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A41:G42"/>
-    <mergeCell ref="B116:G116"/>
+    <mergeCell ref="D113:G113"/>
+    <mergeCell ref="A113:C113"/>
     <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A115:G115"/>
+    <mergeCell ref="A117:G117"/>
+    <mergeCell ref="A13:G13"/>
     <mergeCell ref="B103:G103"/>
-    <mergeCell ref="A111:G111"/>
-    <mergeCell ref="A44:G44"/>
-    <mergeCell ref="B112:G112"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A67:G67"/>
-    <mergeCell ref="A87:G88"/>
+    <mergeCell ref="B99:G99"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="C10:G10"/>
-    <mergeCell ref="B99:G99"/>
-    <mergeCell ref="A24:G24"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B128:G128"/>
+    <mergeCell ref="B118:G118"/>
+    <mergeCell ref="B127:G127"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="B92:G92"/>
-    <mergeCell ref="A37:G38"/>
-    <mergeCell ref="D46:G46"/>
+    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="C9:G9"/>
     <mergeCell ref="B104:G104"/>
-    <mergeCell ref="B124:G124"/>
-    <mergeCell ref="B95:G95"/>
-    <mergeCell ref="A132:G134"/>
-    <mergeCell ref="A119:G119"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="D45:G45"/>
     <mergeCell ref="B123:G123"/>
-    <mergeCell ref="B114:G114"/>
-    <mergeCell ref="B94:G94"/>
-    <mergeCell ref="A33:G34"/>
+    <mergeCell ref="A134:G135"/>
+    <mergeCell ref="B110:G110"/>
     <mergeCell ref="C11:G11"/>
-    <mergeCell ref="D108:G108"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="B113:G113"/>
+    <mergeCell ref="D52:G52"/>
+    <mergeCell ref="A47:G48"/>
+    <mergeCell ref="B126:G126"/>
+    <mergeCell ref="B106:G106"/>
     <mergeCell ref="B97:G97"/>
-    <mergeCell ref="A90:G90"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A114:C114"/>
     <mergeCell ref="B100:G100"/>
-    <mergeCell ref="B91:G91"/>
-    <mergeCell ref="D107:G107"/>
-    <mergeCell ref="B125:G125"/>
-    <mergeCell ref="A107:C107"/>
+    <mergeCell ref="B131:G131"/>
+    <mergeCell ref="B129:G129"/>
+    <mergeCell ref="B109:G109"/>
+    <mergeCell ref="A137:G137"/>
+    <mergeCell ref="A35:G36"/>
+    <mergeCell ref="A93:G94"/>
     <mergeCell ref="B121:G121"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="A27:G27"/>
-    <mergeCell ref="B115:G115"/>
-    <mergeCell ref="A136:G136"/>
+    <mergeCell ref="D53:G53"/>
     <mergeCell ref="A21:G21"/>
-    <mergeCell ref="D47:G47"/>
+    <mergeCell ref="A43:G44"/>
+    <mergeCell ref="B122:G122"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A39:G40"/>
     <mergeCell ref="B102:G102"/>
-    <mergeCell ref="B122:G122"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="B93:G93"/>
+    <mergeCell ref="B105:G105"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B105:G105"/>
-    <mergeCell ref="B96:G96"/>
+    <mergeCell ref="B130:G130"/>
     <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Split staff counts and completions into AM and PM crews
Staff #'s, shift leads, staff to coach (1 Huddl) and 7shifts completion now
appear twice — once for the AM crew and once for the PM crew — for eight
blocks total, since game day turns over mid-shift.

Every field on the web version carries its own am/pm key so the two crews
save independently.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Game Day Pre-Shift" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$137</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.5" customWidth="1" min="1" max="1"/>
@@ -1078,52 +1078,46 @@
       <c r="F54" s="5" t="n"/>
       <c r="G54" s="5" t="n"/>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>AM CREW — STAFF #'S &amp; COMPLETIONS</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="7" t="n"/>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>STAFF #'S</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>SHIFT LEADS:</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>STAFF TO COACH:</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="19" customHeight="1">
-      <c r="A57" s="20" t="inlineStr">
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>SHIFT LEADS</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>STAFF TO COACH — 1 HUDDL</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="20" t="inlineStr">
         <is>
           <t>SERVERS:</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="n"/>
-      <c r="C57" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="n"/>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>1 HUDDL COMPLETION</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="19" customHeight="1">
-      <c r="A58" s="20" t="inlineStr">
-        <is>
-          <t>BARTENDERS:</t>
         </is>
       </c>
       <c r="B58" s="5" t="n"/>
       <c r="C58" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="D58" s="5" t="n"/>
@@ -1133,17 +1127,18 @@
         </is>
       </c>
       <c r="F58" s="5" t="n"/>
-    </row>
-    <row r="59" ht="19" customHeight="1">
+      <c r="G58" s="5" t="n"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>BARTENDERS:</t>
         </is>
       </c>
       <c r="B59" s="5" t="n"/>
       <c r="C59" s="20" t="inlineStr">
         <is>
-          <t>BARTENDER:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="D59" s="5" t="n"/>
@@ -1153,17 +1148,18 @@
         </is>
       </c>
       <c r="F59" s="5" t="n"/>
-    </row>
-    <row r="60" ht="19" customHeight="1">
+      <c r="G59" s="5" t="n"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
         <is>
-          <t>HOSTS:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="B60" s="5" t="n"/>
       <c r="C60" s="20" t="inlineStr">
         <is>
-          <t>HOST:</t>
+          <t>BARTENDER:</t>
         </is>
       </c>
       <c r="D60" s="5" t="n"/>
@@ -1173,17 +1169,18 @@
         </is>
       </c>
       <c r="F60" s="5" t="n"/>
-    </row>
-    <row r="61" ht="19" customHeight="1">
+      <c r="G60" s="5" t="n"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="20" t="inlineStr">
         <is>
-          <t>RUNNERS:</t>
+          <t>HOSTS:</t>
         </is>
       </c>
       <c r="B61" s="5" t="n"/>
       <c r="C61" s="20" t="inlineStr">
         <is>
-          <t>BAR:</t>
+          <t>HOST:</t>
         </is>
       </c>
       <c r="D61" s="5" t="n"/>
@@ -1193,17 +1190,18 @@
         </is>
       </c>
       <c r="F61" s="5" t="n"/>
-    </row>
-    <row r="62" ht="19" customHeight="1">
+      <c r="G61" s="5" t="n"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="20" t="inlineStr">
         <is>
-          <t>BARBACKS:</t>
+          <t>RUNNERS:</t>
         </is>
       </c>
       <c r="B62" s="5" t="n"/>
       <c r="C62" s="20" t="inlineStr">
         <is>
-          <t>BARBACK:</t>
+          <t>BAR:</t>
         </is>
       </c>
       <c r="D62" s="5" t="n"/>
@@ -1213,642 +1211,664 @@
         </is>
       </c>
       <c r="F62" s="5" t="n"/>
-    </row>
-    <row r="63" ht="19" customHeight="1">
+      <c r="G62" s="5" t="n"/>
+    </row>
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="20" t="inlineStr">
         <is>
+          <t>BARBACKS:</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n"/>
+      <c r="C63" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="n"/>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="20" t="inlineStr">
+        <is>
           <t>SHOT GIRL:</t>
         </is>
       </c>
-      <c r="B63" s="5" t="n"/>
-    </row>
-    <row r="64" ht="19" customHeight="1">
-      <c r="A64" s="20" t="inlineStr">
+      <c r="B64" s="5" t="n"/>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="20" t="inlineStr">
         <is>
           <t>MANAGERS:</t>
         </is>
       </c>
-      <c r="B64" s="5" t="n"/>
-    </row>
-    <row r="66">
-      <c r="E66" s="4" t="inlineStr">
+      <c r="B65" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>7SHIFTS COMPLETION</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="E67" s="20" t="inlineStr">
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="20" t="inlineStr">
         <is>
           <t>SERVER:</t>
         </is>
       </c>
-      <c r="F67" s="5" t="n"/>
-    </row>
-    <row r="68">
-      <c r="E68" s="20" t="inlineStr">
+      <c r="B68" s="5" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="20" t="inlineStr">
         <is>
           <t>BAR:</t>
         </is>
       </c>
-      <c r="F68" s="5" t="n"/>
-    </row>
-    <row r="69">
-      <c r="E69" s="20" t="inlineStr">
+      <c r="B69" s="5" t="n"/>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="20" t="inlineStr">
         <is>
           <t>CAFÉ:</t>
         </is>
       </c>
-      <c r="F69" s="5" t="n"/>
-    </row>
-    <row r="70">
-      <c r="E70" s="20" t="inlineStr">
+      <c r="B70" s="5" t="n"/>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="20" t="inlineStr">
         <is>
           <t>HOST:</t>
         </is>
       </c>
-      <c r="F70" s="5" t="n"/>
-    </row>
-    <row r="71">
-      <c r="E71" s="20" t="inlineStr">
+      <c r="B71" s="5" t="n"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="20" t="inlineStr">
         <is>
           <t>BARBACK:</t>
         </is>
       </c>
-      <c r="F71" s="5" t="n"/>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>STATION ASSIGNMENTS — WRITE A NAME ON EVERY LINE</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="n"/>
-      <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
-      <c r="E73" s="7" t="n"/>
-      <c r="F73" s="7" t="n"/>
-      <c r="G73" s="7" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>HOST</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>RUNNERS</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="9" t="inlineStr">
-        <is>
-          <t>Lead:</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="n"/>
-      <c r="C75" s="9" t="inlineStr">
-        <is>
-          <t>Bar 100:</t>
-        </is>
-      </c>
-      <c r="D75" s="5" t="n"/>
-      <c r="E75" s="9" t="inlineStr">
-        <is>
-          <t>100:</t>
-        </is>
-      </c>
-      <c r="F75" s="5" t="n"/>
-      <c r="G75" s="5" t="n"/>
+      <c r="B72" s="5" t="n"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>PM CREW — STAFF #'S &amp; COMPLETIONS</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="n"/>
+      <c r="C74" s="7" t="n"/>
+      <c r="D74" s="7" t="n"/>
+      <c r="E74" s="7" t="n"/>
+      <c r="F74" s="7" t="n"/>
+      <c r="G74" s="7" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>STAFF #'S</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>SHIFT LEADS</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>STAFF TO COACH — 1 HUDDL</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="9" t="inlineStr">
-        <is>
-          <t>Runner:</t>
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>SERVERS:</t>
         </is>
       </c>
       <c r="B76" s="5" t="n"/>
-      <c r="C76" s="9" t="inlineStr">
-        <is>
-          <t>Bar 200:</t>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="D76" s="5" t="n"/>
-      <c r="E76" s="9" t="inlineStr">
-        <is>
-          <t>105:</t>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="F76" s="5" t="n"/>
       <c r="G76" s="5" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="9" t="inlineStr">
-        <is>
-          <t>Waters:</t>
+      <c r="A77" s="20" t="inlineStr">
+        <is>
+          <t>BARTENDERS:</t>
         </is>
       </c>
       <c r="B77" s="5" t="n"/>
-      <c r="C77" s="9" t="inlineStr">
-        <is>
-          <t>Food:</t>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="D77" s="5" t="n"/>
-      <c r="E77" s="9" t="inlineStr">
-        <is>
-          <t>110:</t>
+      <c r="E77" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
         </is>
       </c>
       <c r="F77" s="5" t="n"/>
       <c r="G77" s="5" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="9" t="inlineStr">
-        <is>
-          <t>Bathrooms:</t>
+      <c r="A78" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="B78" s="5" t="n"/>
-      <c r="E78" s="9" t="inlineStr">
-        <is>
-          <t>200:</t>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>BARTENDER:</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="F78" s="5" t="n"/>
       <c r="G78" s="5" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="E79" s="9" t="inlineStr">
-        <is>
-          <t>Patio:</t>
+      <c r="A79" s="20" t="inlineStr">
+        <is>
+          <t>HOSTS:</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="n"/>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="n"/>
+      <c r="E79" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
         </is>
       </c>
       <c r="F79" s="5" t="n"/>
       <c r="G79" s="5" t="n"/>
     </row>
-    <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="20" t="inlineStr">
+        <is>
+          <t>RUNNERS:</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="n"/>
+      <c r="C80" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="n"/>
+      <c r="G80" s="5" t="n"/>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="20" t="inlineStr">
+        <is>
+          <t>BARBACKS:</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="n"/>
+      <c r="C81" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="n"/>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="20" t="inlineStr">
+        <is>
+          <t>SHOT GIRL:</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="n"/>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="20" t="inlineStr">
+        <is>
+          <t>MANAGERS:</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>7SHIFTS COMPLETION</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n"/>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="6" t="inlineStr">
+        <is>
+          <t>STATION ASSIGNMENTS — WRITE A NAME ON EVERY LINE</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="n"/>
+      <c r="C92" s="7" t="n"/>
+      <c r="D92" s="7" t="n"/>
+      <c r="E92" s="7" t="n"/>
+      <c r="F92" s="7" t="n"/>
+      <c r="G92" s="7" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>HOST</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>RUNNERS</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>Lead:</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="n"/>
+      <c r="C94" s="9" t="inlineStr">
+        <is>
+          <t>Bar 100:</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="n"/>
+      <c r="E94" s="9" t="inlineStr">
+        <is>
+          <t>100:</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="n"/>
+      <c r="G94" s="5" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>Runner:</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="n"/>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>Bar 200:</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="n"/>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>105:</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="n"/>
+      <c r="G95" s="5" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>Waters:</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="n"/>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>Food:</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="n"/>
+      <c r="E96" s="9" t="inlineStr">
+        <is>
+          <t>110:</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="n"/>
+      <c r="G96" s="5" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="9" t="inlineStr">
+        <is>
+          <t>Bathrooms:</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="n"/>
+      <c r="E97" s="9" t="inlineStr">
+        <is>
+          <t>200:</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="n"/>
+      <c r="G97" s="5" t="n"/>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t>Patio:</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="n"/>
+      <c r="G98" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
         <is>
           <t>BARBACKS</t>
         </is>
       </c>
-      <c r="C81" s="8" t="inlineStr">
+      <c r="C100" s="8" t="inlineStr">
         <is>
           <t>SHOT GIRL</t>
         </is>
       </c>
-      <c r="E81" s="8" t="inlineStr">
+      <c r="E100" s="8" t="inlineStr">
         <is>
           <t>TASTE PLATE</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="9" t="inlineStr">
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="9" t="inlineStr">
         <is>
           <t>Main Bar:</t>
         </is>
       </c>
-      <c r="B82" s="5" t="n"/>
-      <c r="C82" s="9" t="inlineStr">
+      <c r="B101" s="5" t="n"/>
+      <c r="C101" s="9" t="inlineStr">
         <is>
           <t>On tonight:</t>
         </is>
       </c>
-      <c r="D82" s="5" t="n"/>
-      <c r="E82" s="9" t="inlineStr">
+      <c r="D101" s="5" t="n"/>
+      <c r="E101" s="9" t="inlineStr">
         <is>
           <t>Running it:</t>
         </is>
       </c>
-      <c r="F82" s="5" t="n"/>
-      <c r="G82" s="5" t="n"/>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="9" t="inlineStr">
+      <c r="F101" s="5" t="n"/>
+      <c r="G101" s="5" t="n"/>
+    </row>
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="9" t="inlineStr">
         <is>
           <t>Patio Bar:</t>
         </is>
       </c>
-      <c r="B83" s="5" t="n"/>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="9" t="inlineStr">
+      <c r="B102" s="5" t="n"/>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>Main Floor:</t>
         </is>
       </c>
-      <c r="B84" s="5" t="n"/>
-    </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="9" t="inlineStr">
+      <c r="B103" s="5" t="n"/>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="9" t="inlineStr">
         <is>
           <t>Café:</t>
         </is>
       </c>
-      <c r="B85" s="5" t="n"/>
-    </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="9" t="inlineStr">
+      <c r="B104" s="5" t="n"/>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="9" t="inlineStr">
         <is>
           <t>Front Patio:</t>
         </is>
       </c>
-      <c r="B86" s="5" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="8" t="inlineStr">
+      <c r="B105" s="5" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
         <is>
           <t>SOCIAL MEDIA</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="9" t="inlineStr">
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="9" t="inlineStr">
         <is>
           <t>On tonight:</t>
         </is>
       </c>
-      <c r="B89" s="5" t="n"/>
-    </row>
-    <row r="90" ht="18" customHeight="1">
-      <c r="A90" s="9" t="inlineStr">
+      <c r="B108" s="5" t="n"/>
+    </row>
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="9" t="inlineStr">
         <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B90" s="5" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+      <c r="B109" s="5" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>PARTIES / EVENTS:</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="16" t="n"/>
-      <c r="B93" s="17" t="n"/>
-      <c r="C93" s="17" t="n"/>
-      <c r="D93" s="17" t="n"/>
-      <c r="E93" s="17" t="n"/>
-      <c r="F93" s="17" t="n"/>
-      <c r="G93" s="17" t="n"/>
-    </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="17" t="n"/>
-      <c r="B94" s="17" t="n"/>
-      <c r="C94" s="17" t="n"/>
-      <c r="D94" s="17" t="n"/>
-      <c r="E94" s="17" t="n"/>
-      <c r="F94" s="17" t="n"/>
-      <c r="G94" s="17" t="n"/>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="6" t="inlineStr">
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="16" t="n"/>
+      <c r="B112" s="17" t="n"/>
+      <c r="C112" s="17" t="n"/>
+      <c r="D112" s="17" t="n"/>
+      <c r="E112" s="17" t="n"/>
+      <c r="F112" s="17" t="n"/>
+      <c r="G112" s="17" t="n"/>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="17" t="n"/>
+      <c r="B113" s="17" t="n"/>
+      <c r="C113" s="17" t="n"/>
+      <c r="D113" s="17" t="n"/>
+      <c r="E113" s="17" t="n"/>
+      <c r="F113" s="17" t="n"/>
+      <c r="G113" s="17" t="n"/>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="6" t="inlineStr">
         <is>
           <t>GAME DAY OPEN — 90 MINUTES BEFORE DOORS</t>
         </is>
       </c>
-      <c r="B96" s="7" t="n"/>
-      <c r="C96" s="7" t="n"/>
-      <c r="D96" s="7" t="n"/>
-      <c r="E96" s="7" t="n"/>
-      <c r="F96" s="7" t="n"/>
-      <c r="G96" s="7" t="n"/>
-    </row>
-    <row r="97" ht="17" customHeight="1">
-      <c r="A97" s="21" t="inlineStr">
+      <c r="B115" s="7" t="n"/>
+      <c r="C115" s="7" t="n"/>
+      <c r="D115" s="7" t="n"/>
+      <c r="E115" s="7" t="n"/>
+      <c r="F115" s="7" t="n"/>
+      <c r="G115" s="7" t="n"/>
+    </row>
+    <row r="116" ht="17" customHeight="1">
+      <c r="A116" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B97" s="9" t="inlineStr">
+      <c r="B116" s="9" t="inlineStr">
         <is>
           <t>Know the game — kickoff, attendance, national TV, weather. Times on the board.</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="17" customHeight="1">
-      <c r="A98" s="21" t="inlineStr">
+    <row r="117" ht="17" customHeight="1">
+      <c r="A117" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B98" s="9" t="inlineStr">
+      <c r="B117" s="9" t="inlineStr">
         <is>
           <t>Every staff member can name all three promos — ask two people at random before pre-shift ends.</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="17" customHeight="1">
-      <c r="A99" s="21" t="inlineStr">
+    <row r="118" ht="17" customHeight="1">
+      <c r="A118" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B99" s="9" t="inlineStr">
+      <c r="B118" s="9" t="inlineStr">
         <is>
           <t>Anthem time on the board — every staff member knows to line up behind the bar.</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="17" customHeight="1">
-      <c r="A100" s="21" t="inlineStr">
+    <row r="119" ht="17" customHeight="1">
+      <c r="A119" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B100" s="9" t="inlineStr">
+      <c r="B119" s="9" t="inlineStr">
         <is>
           <t>Social media assigned, phone charged, and they know the shot list.</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="17" customHeight="1">
-      <c r="A101" s="21" t="inlineStr">
+    <row r="120" ht="17" customHeight="1">
+      <c r="A120" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B101" s="9" t="inlineStr">
+      <c r="B120" s="9" t="inlineStr">
         <is>
           <t>Three windows built on paper — cut times, breaks, post-game all-hands decided now.</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="17" customHeight="1">
-      <c r="A102" s="21" t="inlineStr">
+    <row r="121" ht="17" customHeight="1">
+      <c r="A121" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B102" s="9" t="inlineStr">
+      <c r="B121" s="9" t="inlineStr">
         <is>
           <t>Staffing confirmed against 7shifts. One no-show on game day is a two-hour wait.</t>
         </is>
       </c>
     </row>
-    <row r="103" ht="17" customHeight="1">
-      <c r="A103" s="21" t="inlineStr">
+    <row r="122" ht="17" customHeight="1">
+      <c r="A122" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B103" s="9" t="inlineStr">
+      <c r="B122" s="9" t="inlineStr">
         <is>
           <t>Every station walked, front and back. The 3 Rules on all of them.</t>
         </is>
       </c>
     </row>
-    <row r="104" ht="17" customHeight="1">
-      <c r="A104" s="21" t="inlineStr">
+    <row r="123" ht="17" customHeight="1">
+      <c r="A123" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B104" s="9" t="inlineStr">
+      <c r="B123" s="9" t="inlineStr">
         <is>
           <t>Bar par DOUBLED — ice, kegs, backups, garnish, glassware, batch.</t>
         </is>
       </c>
     </row>
-    <row r="105" ht="17" customHeight="1">
-      <c r="A105" s="21" t="inlineStr">
+    <row r="124" ht="17" customHeight="1">
+      <c r="A124" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B105" s="9" t="inlineStr">
+      <c r="B124" s="9" t="inlineStr">
         <is>
           <t>86 board walked with the kitchen, current and visible.</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="17" customHeight="1">
-      <c r="A106" s="21" t="inlineStr">
+    <row r="125" ht="17" customHeight="1">
+      <c r="A125" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B106" s="9" t="inlineStr">
+      <c r="B125" s="9" t="inlineStr">
         <is>
           <t>TVs, sound and the game feed tested before a single guest sits down.</t>
         </is>
       </c>
-    </row>
-    <row r="107" ht="17" customHeight="1">
-      <c r="A107" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B107" s="9" t="inlineStr">
-        <is>
-          <t>ID check covered — door and bar know who is carding, and the light works.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="17" customHeight="1">
-      <c r="A108" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B108" s="9" t="inlineStr">
-        <is>
-          <t>Restrooms stocked and clean before doors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="17" customHeight="1">
-      <c r="A109" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B109" s="9" t="inlineStr">
-        <is>
-          <t>POS, printers and card processing tested with a live ticket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="17" customHeight="1">
-      <c r="A110" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B110" s="9" t="inlineStr">
-        <is>
-          <t>Cash on hand for a bar that will run cash all night.</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="17" customHeight="1">
-      <c r="A111" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B111" s="9" t="inlineStr">
-        <is>
-          <t>Door, patio and line plan — where the wait forms and who holds it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="22" t="inlineStr">
-        <is>
-          <t>IS STAFF IN UNIFORM?   YES / NO</t>
-        </is>
-      </c>
-      <c r="B113" s="13" t="n"/>
-      <c r="C113" s="13" t="n"/>
-      <c r="D113" s="22" t="inlineStr">
-        <is>
-          <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
-        </is>
-      </c>
-      <c r="E113" s="13" t="n"/>
-      <c r="F113" s="13" t="n"/>
-      <c r="G113" s="13" t="n"/>
-    </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="22" t="inlineStr">
-        <is>
-          <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
-        </is>
-      </c>
-      <c r="B114" s="13" t="n"/>
-      <c r="C114" s="13" t="n"/>
-      <c r="D114" s="22" t="inlineStr">
-        <is>
-          <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
-        </is>
-      </c>
-      <c r="E114" s="13" t="n"/>
-      <c r="F114" s="13" t="n"/>
-      <c r="G114" s="13" t="n"/>
-    </row>
-    <row r="115" ht="20" customHeight="1">
-      <c r="A115" s="22" t="inlineStr">
-        <is>
-          <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
-        </is>
-      </c>
-      <c r="B115" s="13" t="n"/>
-      <c r="C115" s="13" t="n"/>
-      <c r="D115" s="13" t="n"/>
-      <c r="E115" s="13" t="n"/>
-      <c r="F115" s="13" t="n"/>
-      <c r="G115" s="13" t="n"/>
-    </row>
-    <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="6" t="inlineStr">
-        <is>
-          <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
-        </is>
-      </c>
-      <c r="B117" s="7" t="n"/>
-      <c r="C117" s="7" t="n"/>
-      <c r="D117" s="7" t="n"/>
-      <c r="E117" s="7" t="n"/>
-      <c r="F117" s="7" t="n"/>
-      <c r="G117" s="7" t="n"/>
-    </row>
-    <row r="118" ht="32" customHeight="1">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B118" s="9" t="inlineStr">
-        <is>
-          <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="32" customHeight="1">
-      <c r="A119" s="8" t="inlineStr">
-        <is>
-          <t>SERVERS</t>
-        </is>
-      </c>
-      <c r="B119" s="9" t="inlineStr">
-        <is>
-          <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="32" customHeight="1">
-      <c r="A120" s="8" t="inlineStr">
-        <is>
-          <t>HOST</t>
-        </is>
-      </c>
-      <c r="B120" s="9" t="inlineStr">
-        <is>
-          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. Card at the door when the room is young; it is far easier there than at the bar. Keep the line off the sidewalk and feed the wait to the bar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="32" customHeight="1">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t>KITCHEN</t>
-        </is>
-      </c>
-      <c r="B121" s="9" t="inlineStr">
-        <is>
-          <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="32" customHeight="1">
-      <c r="A122" s="8" t="inlineStr">
-        <is>
-          <t>SOCIAL</t>
-        </is>
-      </c>
-      <c r="B122" s="9" t="inlineStr">
-        <is>
-          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="32" customHeight="1">
-      <c r="A123" s="8" t="inlineStr">
-        <is>
-          <t>SUPPORT</t>
-        </is>
-      </c>
-      <c r="B123" s="9" t="inlineStr">
-        <is>
-          <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="18" customHeight="1">
-      <c r="A125" s="6" t="inlineStr">
-        <is>
-          <t>POST-GAME &amp; CLOSE</t>
-        </is>
-      </c>
-      <c r="B125" s="7" t="n"/>
-      <c r="C125" s="7" t="n"/>
-      <c r="D125" s="7" t="n"/>
-      <c r="E125" s="7" t="n"/>
-      <c r="F125" s="7" t="n"/>
-      <c r="G125" s="7" t="n"/>
     </row>
     <row r="126" ht="17" customHeight="1">
       <c r="A126" s="21" t="inlineStr">
@@ -1858,7 +1878,7 @@
       </c>
       <c r="B126" s="9" t="inlineStr">
         <is>
-          <t>All hands on the floor BEFORE the final whistle — not after.</t>
+          <t>ID check covered — door and bar know who is carding, and the light works.</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1890,7 @@
       </c>
       <c r="B127" s="9" t="inlineStr">
         <is>
-          <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
+          <t>Restrooms stocked and clean before doors.</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1902,7 @@
       </c>
       <c r="B128" s="9" t="inlineStr">
         <is>
-          <t>Every void, comp and discount reconciled to a manager name.</t>
+          <t>POS, printers and card processing tested with a live ticket.</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1914,7 @@
       </c>
       <c r="B129" s="9" t="inlineStr">
         <is>
-          <t>Every refusal or cut-off logged with what happened and who made the call.</t>
+          <t>Cash on hand for a bar that will run cash all night.</t>
         </is>
       </c>
     </row>
@@ -1906,124 +1926,331 @@
       </c>
       <c r="B130" s="9" t="inlineStr">
         <is>
+          <t>Door, patio and line plan — where the wait forms and who holds it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="20" customHeight="1">
+      <c r="A132" s="22" t="inlineStr">
+        <is>
+          <t>IS STAFF IN UNIFORM?   YES / NO</t>
+        </is>
+      </c>
+      <c r="B132" s="13" t="n"/>
+      <c r="C132" s="13" t="n"/>
+      <c r="D132" s="22" t="inlineStr">
+        <is>
+          <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
+        </is>
+      </c>
+      <c r="E132" s="13" t="n"/>
+      <c r="F132" s="13" t="n"/>
+      <c r="G132" s="13" t="n"/>
+    </row>
+    <row r="133" ht="20" customHeight="1">
+      <c r="A133" s="22" t="inlineStr">
+        <is>
+          <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
+        </is>
+      </c>
+      <c r="B133" s="13" t="n"/>
+      <c r="C133" s="13" t="n"/>
+      <c r="D133" s="22" t="inlineStr">
+        <is>
+          <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
+        </is>
+      </c>
+      <c r="E133" s="13" t="n"/>
+      <c r="F133" s="13" t="n"/>
+      <c r="G133" s="13" t="n"/>
+    </row>
+    <row r="134" ht="20" customHeight="1">
+      <c r="A134" s="22" t="inlineStr">
+        <is>
+          <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
+        </is>
+      </c>
+      <c r="B134" s="13" t="n"/>
+      <c r="C134" s="13" t="n"/>
+      <c r="D134" s="13" t="n"/>
+      <c r="E134" s="13" t="n"/>
+      <c r="F134" s="13" t="n"/>
+      <c r="G134" s="13" t="n"/>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="6" t="inlineStr">
+        <is>
+          <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
+        </is>
+      </c>
+      <c r="B136" s="7" t="n"/>
+      <c r="C136" s="7" t="n"/>
+      <c r="D136" s="7" t="n"/>
+      <c r="E136" s="7" t="n"/>
+      <c r="F136" s="7" t="n"/>
+      <c r="G136" s="7" t="n"/>
+    </row>
+    <row r="137" ht="32" customHeight="1">
+      <c r="A137" s="8" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="B137" s="9" t="inlineStr">
+        <is>
+          <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="32" customHeight="1">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t>SERVERS</t>
+        </is>
+      </c>
+      <c r="B138" s="9" t="inlineStr">
+        <is>
+          <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="32" customHeight="1">
+      <c r="A139" s="8" t="inlineStr">
+        <is>
+          <t>HOST</t>
+        </is>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. Card at the door when the room is young; it is far easier there than at the bar. Keep the line off the sidewalk and feed the wait to the bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="32" customHeight="1">
+      <c r="A140" s="8" t="inlineStr">
+        <is>
+          <t>KITCHEN</t>
+        </is>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
+        <is>
+          <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="32" customHeight="1">
+      <c r="A141" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL</t>
+        </is>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="32" customHeight="1">
+      <c r="A142" s="8" t="inlineStr">
+        <is>
+          <t>SUPPORT</t>
+        </is>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
+        <is>
+          <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>POST-GAME &amp; CLOSE</t>
+        </is>
+      </c>
+      <c r="B144" s="7" t="n"/>
+      <c r="C144" s="7" t="n"/>
+      <c r="D144" s="7" t="n"/>
+      <c r="E144" s="7" t="n"/>
+      <c r="F144" s="7" t="n"/>
+      <c r="G144" s="7" t="n"/>
+    </row>
+    <row r="145" ht="17" customHeight="1">
+      <c r="A145" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>All hands on the floor BEFORE the final whistle — not after.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="17" customHeight="1">
+      <c r="A146" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="17" customHeight="1">
+      <c r="A147" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>Every void, comp and discount reconciled to a manager name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="17" customHeight="1">
+      <c r="A148" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>Every refusal or cut-off logged with what happened and who made the call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="17" customHeight="1">
+      <c r="A149" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
           <t>Every station back to original position, original condition.</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="17" customHeight="1">
-      <c r="A131" s="21" t="inlineStr">
+    <row r="150" ht="17" customHeight="1">
+      <c r="A150" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B131" s="9" t="inlineStr">
+      <c r="B150" s="9" t="inlineStr">
         <is>
           <t>Shift notes written: what we ran out of, where the wait broke down, what changes next game.</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="4" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
         <is>
           <t>MARKETING:</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="16" t="n"/>
-      <c r="B134" s="17" t="n"/>
-      <c r="C134" s="17" t="n"/>
-      <c r="D134" s="17" t="n"/>
-      <c r="E134" s="17" t="n"/>
-      <c r="F134" s="17" t="n"/>
-      <c r="G134" s="17" t="n"/>
-    </row>
-    <row r="135" ht="18" customHeight="1">
-      <c r="A135" s="17" t="n"/>
-      <c r="B135" s="17" t="n"/>
-      <c r="C135" s="17" t="n"/>
-      <c r="D135" s="17" t="n"/>
-      <c r="E135" s="17" t="n"/>
-      <c r="F135" s="17" t="n"/>
-      <c r="G135" s="17" t="n"/>
-    </row>
-    <row r="137" ht="28" customHeight="1">
-      <c r="A137" s="23" t="inlineStr">
+    <row r="153" ht="18" customHeight="1">
+      <c r="A153" s="16" t="n"/>
+      <c r="B153" s="17" t="n"/>
+      <c r="C153" s="17" t="n"/>
+      <c r="D153" s="17" t="n"/>
+      <c r="E153" s="17" t="n"/>
+      <c r="F153" s="17" t="n"/>
+      <c r="G153" s="17" t="n"/>
+    </row>
+    <row r="154" ht="18" customHeight="1">
+      <c r="A154" s="17" t="n"/>
+      <c r="B154" s="17" t="n"/>
+      <c r="C154" s="17" t="n"/>
+      <c r="D154" s="17" t="n"/>
+      <c r="E154" s="17" t="n"/>
+      <c r="F154" s="17" t="n"/>
+      <c r="G154" s="17" t="n"/>
+    </row>
+    <row r="156" ht="28" customHeight="1">
+      <c r="A156" s="23" t="inlineStr">
         <is>
           <t>100% of our standards, 100% of the time, at 100% volume. A full house is not an excuse to run at 80% — it is the reason we hold the line.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="69">
+  <mergeCells count="71">
     <mergeCell ref="C16:E16"/>
+    <mergeCell ref="B117:G117"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="B120:G120"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="B111:G111"/>
-    <mergeCell ref="B107:G107"/>
-    <mergeCell ref="B101:G101"/>
+    <mergeCell ref="B145:G145"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="B98:G98"/>
-    <mergeCell ref="D114:G114"/>
+    <mergeCell ref="A133:C133"/>
+    <mergeCell ref="A144:G144"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A96:G96"/>
-    <mergeCell ref="A125:G125"/>
+    <mergeCell ref="B148:G148"/>
+    <mergeCell ref="A156:G156"/>
+    <mergeCell ref="A153:G154"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="B119:G119"/>
+    <mergeCell ref="A134:G134"/>
     <mergeCell ref="D51:G51"/>
     <mergeCell ref="A19:G19"/>
-    <mergeCell ref="D113:G113"/>
-    <mergeCell ref="A113:C113"/>
+    <mergeCell ref="B116:G116"/>
+    <mergeCell ref="D133:G133"/>
+    <mergeCell ref="B147:G147"/>
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="A115:G115"/>
-    <mergeCell ref="A117:G117"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="B103:G103"/>
-    <mergeCell ref="B99:G99"/>
+    <mergeCell ref="D132:G132"/>
+    <mergeCell ref="B137:G137"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C10:G10"/>
-    <mergeCell ref="B108:G108"/>
     <mergeCell ref="B128:G128"/>
+    <mergeCell ref="B146:G146"/>
     <mergeCell ref="B118:G118"/>
+    <mergeCell ref="A92:G92"/>
     <mergeCell ref="B127:G127"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A73:G73"/>
     <mergeCell ref="C9:G9"/>
-    <mergeCell ref="B104:G104"/>
+    <mergeCell ref="B139:G139"/>
+    <mergeCell ref="B124:G124"/>
+    <mergeCell ref="B142:G142"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B123:G123"/>
-    <mergeCell ref="A134:G135"/>
-    <mergeCell ref="B110:G110"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="A47:G48"/>
     <mergeCell ref="B126:G126"/>
-    <mergeCell ref="B106:G106"/>
-    <mergeCell ref="B97:G97"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A114:C114"/>
-    <mergeCell ref="B100:G100"/>
-    <mergeCell ref="B131:G131"/>
+    <mergeCell ref="A112:G113"/>
+    <mergeCell ref="B138:G138"/>
     <mergeCell ref="B129:G129"/>
-    <mergeCell ref="B109:G109"/>
-    <mergeCell ref="A137:G137"/>
     <mergeCell ref="A35:G36"/>
-    <mergeCell ref="A93:G94"/>
+    <mergeCell ref="B125:G125"/>
+    <mergeCell ref="A74:G74"/>
     <mergeCell ref="B121:G121"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A56:G56"/>
     <mergeCell ref="D53:G53"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A43:G44"/>
     <mergeCell ref="B122:G122"/>
     <mergeCell ref="A50:G50"/>
     <mergeCell ref="A39:G40"/>
-    <mergeCell ref="B102:G102"/>
+    <mergeCell ref="A132:C132"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="B105:G105"/>
+    <mergeCell ref="A136:G136"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B140:G140"/>
+    <mergeCell ref="B149:G149"/>
+    <mergeCell ref="B150:G150"/>
     <mergeCell ref="B130:G130"/>
+    <mergeCell ref="B141:G141"/>
     <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Split station assignments into AM and PM crews
Host, Runners, Bar, Barbacks, Shot girl, Taste plate and Social media each
appear twice — once per crew, fourteen blocks total — matching the AM/PM
split already applied to staff counts and completions.

Replaces the one-off station layout with the shared stack_group helper, so
both sections build from the same code.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Game Day Pre-Shift" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$156</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$178</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G156"/>
+  <dimension ref="A1:G178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.5" customWidth="1" min="1" max="1"/>
@@ -1515,565 +1515,535 @@
       <c r="F92" s="7" t="n"/>
       <c r="G92" s="7" t="n"/>
     </row>
-    <row r="93">
+    <row r="93" ht="17" customHeight="1">
       <c r="A93" s="8" t="inlineStr">
         <is>
+          <t>AM CREW</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
           <t>HOST</t>
         </is>
       </c>
-      <c r="C93" s="8" t="inlineStr">
+      <c r="C94" s="8" t="inlineStr">
         <is>
           <t>RUNNERS</t>
         </is>
       </c>
-      <c r="E93" s="8" t="inlineStr">
+      <c r="E94" s="8" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="9" t="inlineStr">
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="20" t="inlineStr">
         <is>
           <t>Lead:</t>
         </is>
       </c>
-      <c r="B94" s="5" t="n"/>
-      <c r="C94" s="9" t="inlineStr">
+      <c r="B95" s="5" t="n"/>
+      <c r="C95" s="20" t="inlineStr">
         <is>
           <t>Bar 100:</t>
         </is>
       </c>
-      <c r="D94" s="5" t="n"/>
-      <c r="E94" s="9" t="inlineStr">
+      <c r="D95" s="5" t="n"/>
+      <c r="E95" s="20" t="inlineStr">
         <is>
           <t>100:</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="n"/>
-      <c r="G94" s="5" t="n"/>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="9" t="inlineStr">
-        <is>
-          <t>Runner:</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="n"/>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>Bar 200:</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="n"/>
-      <c r="E95" s="9" t="inlineStr">
-        <is>
-          <t>105:</t>
         </is>
       </c>
       <c r="F95" s="5" t="n"/>
       <c r="G95" s="5" t="n"/>
     </row>
     <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="9" t="inlineStr">
-        <is>
-          <t>Waters:</t>
+      <c r="A96" s="20" t="inlineStr">
+        <is>
+          <t>Runner:</t>
         </is>
       </c>
       <c r="B96" s="5" t="n"/>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>Food:</t>
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>Bar 200:</t>
         </is>
       </c>
       <c r="D96" s="5" t="n"/>
-      <c r="E96" s="9" t="inlineStr">
-        <is>
-          <t>110:</t>
+      <c r="E96" s="20" t="inlineStr">
+        <is>
+          <t>105:</t>
         </is>
       </c>
       <c r="F96" s="5" t="n"/>
       <c r="G96" s="5" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="9" t="inlineStr">
-        <is>
-          <t>Bathrooms:</t>
+      <c r="A97" s="20" t="inlineStr">
+        <is>
+          <t>Waters:</t>
         </is>
       </c>
       <c r="B97" s="5" t="n"/>
-      <c r="E97" s="9" t="inlineStr">
-        <is>
-          <t>200:</t>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>Food:</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="n"/>
+      <c r="E97" s="20" t="inlineStr">
+        <is>
+          <t>110:</t>
         </is>
       </c>
       <c r="F97" s="5" t="n"/>
       <c r="G97" s="5" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
-      <c r="E98" s="9" t="inlineStr">
-        <is>
-          <t>Patio:</t>
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t>Bathrooms:</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="n"/>
+      <c r="E98" s="20" t="inlineStr">
+        <is>
+          <t>200:</t>
         </is>
       </c>
       <c r="F98" s="5" t="n"/>
       <c r="G98" s="5" t="n"/>
     </row>
-    <row r="100">
-      <c r="A100" s="8" t="inlineStr">
+    <row r="99" ht="18" customHeight="1">
+      <c r="E99" s="20" t="inlineStr">
+        <is>
+          <t>Patio:</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="n"/>
+      <c r="G99" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
         <is>
           <t>BARBACKS</t>
         </is>
       </c>
-      <c r="C100" s="8" t="inlineStr">
+      <c r="C101" s="8" t="inlineStr">
         <is>
           <t>SHOT GIRL</t>
         </is>
       </c>
-      <c r="E100" s="8" t="inlineStr">
+      <c r="E101" s="8" t="inlineStr">
         <is>
           <t>TASTE PLATE</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="9" t="inlineStr">
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="20" t="inlineStr">
         <is>
           <t>Main Bar:</t>
         </is>
       </c>
-      <c r="B101" s="5" t="n"/>
-      <c r="C101" s="9" t="inlineStr">
+      <c r="B102" s="5" t="n"/>
+      <c r="C102" s="20" t="inlineStr">
         <is>
           <t>On tonight:</t>
         </is>
       </c>
-      <c r="D101" s="5" t="n"/>
-      <c r="E101" s="9" t="inlineStr">
+      <c r="D102" s="5" t="n"/>
+      <c r="E102" s="20" t="inlineStr">
         <is>
           <t>Running it:</t>
         </is>
       </c>
-      <c r="F101" s="5" t="n"/>
-      <c r="G101" s="5" t="n"/>
-    </row>
-    <row r="102" ht="18" customHeight="1">
-      <c r="A102" s="9" t="inlineStr">
+      <c r="F102" s="5" t="n"/>
+      <c r="G102" s="5" t="n"/>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="20" t="inlineStr">
         <is>
           <t>Patio Bar:</t>
         </is>
       </c>
-      <c r="B102" s="5" t="n"/>
-    </row>
-    <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="9" t="inlineStr">
+      <c r="B103" s="5" t="n"/>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="20" t="inlineStr">
         <is>
           <t>Main Floor:</t>
         </is>
       </c>
-      <c r="B103" s="5" t="n"/>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="9" t="inlineStr">
+      <c r="B104" s="5" t="n"/>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="20" t="inlineStr">
         <is>
           <t>Café:</t>
         </is>
       </c>
-      <c r="B104" s="5" t="n"/>
-    </row>
-    <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="9" t="inlineStr">
+      <c r="B105" s="5" t="n"/>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="20" t="inlineStr">
         <is>
           <t>Front Patio:</t>
         </is>
       </c>
-      <c r="B105" s="5" t="n"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="8" t="inlineStr">
+      <c r="B106" s="5" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
         <is>
           <t>SOCIAL MEDIA</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="9" t="inlineStr">
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="20" t="inlineStr">
         <is>
           <t>On tonight:</t>
         </is>
       </c>
-      <c r="B108" s="5" t="n"/>
-    </row>
-    <row r="109" ht="18" customHeight="1">
-      <c r="A109" s="9" t="inlineStr">
+      <c r="B109" s="5" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="20" t="inlineStr">
         <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B109" s="5" t="n"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="4" t="inlineStr">
+      <c r="B110" s="5" t="n"/>
+    </row>
+    <row r="113" ht="17" customHeight="1">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>PM CREW</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>HOST</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>RUNNERS</t>
+        </is>
+      </c>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="20" t="inlineStr">
+        <is>
+          <t>Lead:</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="n"/>
+      <c r="C115" s="20" t="inlineStr">
+        <is>
+          <t>Bar 100:</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="n"/>
+      <c r="E115" s="20" t="inlineStr">
+        <is>
+          <t>100:</t>
+        </is>
+      </c>
+      <c r="F115" s="5" t="n"/>
+      <c r="G115" s="5" t="n"/>
+    </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="A116" s="20" t="inlineStr">
+        <is>
+          <t>Runner:</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="n"/>
+      <c r="C116" s="20" t="inlineStr">
+        <is>
+          <t>Bar 200:</t>
+        </is>
+      </c>
+      <c r="D116" s="5" t="n"/>
+      <c r="E116" s="20" t="inlineStr">
+        <is>
+          <t>105:</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="n"/>
+      <c r="G116" s="5" t="n"/>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="20" t="inlineStr">
+        <is>
+          <t>Waters:</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="n"/>
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t>Food:</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="n"/>
+      <c r="E117" s="20" t="inlineStr">
+        <is>
+          <t>110:</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="n"/>
+      <c r="G117" s="5" t="n"/>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="20" t="inlineStr">
+        <is>
+          <t>Bathrooms:</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="n"/>
+      <c r="E118" s="20" t="inlineStr">
+        <is>
+          <t>200:</t>
+        </is>
+      </c>
+      <c r="F118" s="5" t="n"/>
+      <c r="G118" s="5" t="n"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="E119" s="20" t="inlineStr">
+        <is>
+          <t>Patio:</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="n"/>
+      <c r="G119" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t>BARBACKS</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>SHOT GIRL</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>TASTE PLATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="18" customHeight="1">
+      <c r="A122" s="20" t="inlineStr">
+        <is>
+          <t>Main Bar:</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="n"/>
+      <c r="C122" s="20" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="D122" s="5" t="n"/>
+      <c r="E122" s="20" t="inlineStr">
+        <is>
+          <t>Running it:</t>
+        </is>
+      </c>
+      <c r="F122" s="5" t="n"/>
+      <c r="G122" s="5" t="n"/>
+    </row>
+    <row r="123" ht="18" customHeight="1">
+      <c r="A123" s="20" t="inlineStr">
+        <is>
+          <t>Patio Bar:</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="n"/>
+    </row>
+    <row r="124" ht="18" customHeight="1">
+      <c r="A124" s="20" t="inlineStr">
+        <is>
+          <t>Main Floor:</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="n"/>
+    </row>
+    <row r="125" ht="18" customHeight="1">
+      <c r="A125" s="20" t="inlineStr">
+        <is>
+          <t>Café:</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="n"/>
+    </row>
+    <row r="126" ht="18" customHeight="1">
+      <c r="A126" s="20" t="inlineStr">
+        <is>
+          <t>Front Patio:</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL MEDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="18" customHeight="1">
+      <c r="A129" s="20" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="n"/>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="A130" s="20" t="inlineStr">
+        <is>
+          <t>Backup / 2nd half:</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
         <is>
           <t>PARTIES / EVENTS:</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="16" t="n"/>
-      <c r="B112" s="17" t="n"/>
-      <c r="C112" s="17" t="n"/>
-      <c r="D112" s="17" t="n"/>
-      <c r="E112" s="17" t="n"/>
-      <c r="F112" s="17" t="n"/>
-      <c r="G112" s="17" t="n"/>
-    </row>
-    <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="17" t="n"/>
-      <c r="B113" s="17" t="n"/>
-      <c r="C113" s="17" t="n"/>
-      <c r="D113" s="17" t="n"/>
-      <c r="E113" s="17" t="n"/>
-      <c r="F113" s="17" t="n"/>
-      <c r="G113" s="17" t="n"/>
-    </row>
-    <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="6" t="inlineStr">
+    <row r="134" ht="18" customHeight="1">
+      <c r="A134" s="16" t="n"/>
+      <c r="B134" s="17" t="n"/>
+      <c r="C134" s="17" t="n"/>
+      <c r="D134" s="17" t="n"/>
+      <c r="E134" s="17" t="n"/>
+      <c r="F134" s="17" t="n"/>
+      <c r="G134" s="17" t="n"/>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="17" t="n"/>
+      <c r="B135" s="17" t="n"/>
+      <c r="C135" s="17" t="n"/>
+      <c r="D135" s="17" t="n"/>
+      <c r="E135" s="17" t="n"/>
+      <c r="F135" s="17" t="n"/>
+      <c r="G135" s="17" t="n"/>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="A137" s="6" t="inlineStr">
         <is>
           <t>GAME DAY OPEN — 90 MINUTES BEFORE DOORS</t>
         </is>
       </c>
-      <c r="B115" s="7" t="n"/>
-      <c r="C115" s="7" t="n"/>
-      <c r="D115" s="7" t="n"/>
-      <c r="E115" s="7" t="n"/>
-      <c r="F115" s="7" t="n"/>
-      <c r="G115" s="7" t="n"/>
-    </row>
-    <row r="116" ht="17" customHeight="1">
-      <c r="A116" s="21" t="inlineStr">
+      <c r="B137" s="7" t="n"/>
+      <c r="C137" s="7" t="n"/>
+      <c r="D137" s="7" t="n"/>
+      <c r="E137" s="7" t="n"/>
+      <c r="F137" s="7" t="n"/>
+      <c r="G137" s="7" t="n"/>
+    </row>
+    <row r="138" ht="17" customHeight="1">
+      <c r="A138" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B116" s="9" t="inlineStr">
+      <c r="B138" s="9" t="inlineStr">
         <is>
           <t>Know the game — kickoff, attendance, national TV, weather. Times on the board.</t>
         </is>
       </c>
     </row>
-    <row r="117" ht="17" customHeight="1">
-      <c r="A117" s="21" t="inlineStr">
+    <row r="139" ht="17" customHeight="1">
+      <c r="A139" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B117" s="9" t="inlineStr">
+      <c r="B139" s="9" t="inlineStr">
         <is>
           <t>Every staff member can name all three promos — ask two people at random before pre-shift ends.</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="17" customHeight="1">
-      <c r="A118" s="21" t="inlineStr">
+    <row r="140" ht="17" customHeight="1">
+      <c r="A140" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B118" s="9" t="inlineStr">
+      <c r="B140" s="9" t="inlineStr">
         <is>
           <t>Anthem time on the board — every staff member knows to line up behind the bar.</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="17" customHeight="1">
-      <c r="A119" s="21" t="inlineStr">
+    <row r="141" ht="17" customHeight="1">
+      <c r="A141" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B119" s="9" t="inlineStr">
+      <c r="B141" s="9" t="inlineStr">
         <is>
           <t>Social media assigned, phone charged, and they know the shot list.</t>
         </is>
       </c>
     </row>
-    <row r="120" ht="17" customHeight="1">
-      <c r="A120" s="21" t="inlineStr">
+    <row r="142" ht="17" customHeight="1">
+      <c r="A142" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B120" s="9" t="inlineStr">
+      <c r="B142" s="9" t="inlineStr">
         <is>
           <t>Three windows built on paper — cut times, breaks, post-game all-hands decided now.</t>
         </is>
       </c>
     </row>
-    <row r="121" ht="17" customHeight="1">
-      <c r="A121" s="21" t="inlineStr">
+    <row r="143" ht="17" customHeight="1">
+      <c r="A143" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B121" s="9" t="inlineStr">
+      <c r="B143" s="9" t="inlineStr">
         <is>
           <t>Staffing confirmed against 7shifts. One no-show on game day is a two-hour wait.</t>
         </is>
       </c>
     </row>
-    <row r="122" ht="17" customHeight="1">
-      <c r="A122" s="21" t="inlineStr">
+    <row r="144" ht="17" customHeight="1">
+      <c r="A144" s="21" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B122" s="9" t="inlineStr">
+      <c r="B144" s="9" t="inlineStr">
         <is>
           <t>Every station walked, front and back. The 3 Rules on all of them.</t>
         </is>
       </c>
-    </row>
-    <row r="123" ht="17" customHeight="1">
-      <c r="A123" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B123" s="9" t="inlineStr">
-        <is>
-          <t>Bar par DOUBLED — ice, kegs, backups, garnish, glassware, batch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="17" customHeight="1">
-      <c r="A124" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B124" s="9" t="inlineStr">
-        <is>
-          <t>86 board walked with the kitchen, current and visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="17" customHeight="1">
-      <c r="A125" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B125" s="9" t="inlineStr">
-        <is>
-          <t>TVs, sound and the game feed tested before a single guest sits down.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="17" customHeight="1">
-      <c r="A126" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B126" s="9" t="inlineStr">
-        <is>
-          <t>ID check covered — door and bar know who is carding, and the light works.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="17" customHeight="1">
-      <c r="A127" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B127" s="9" t="inlineStr">
-        <is>
-          <t>Restrooms stocked and clean before doors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="17" customHeight="1">
-      <c r="A128" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B128" s="9" t="inlineStr">
-        <is>
-          <t>POS, printers and card processing tested with a live ticket.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="17" customHeight="1">
-      <c r="A129" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B129" s="9" t="inlineStr">
-        <is>
-          <t>Cash on hand for a bar that will run cash all night.</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="17" customHeight="1">
-      <c r="A130" s="21" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B130" s="9" t="inlineStr">
-        <is>
-          <t>Door, patio and line plan — where the wait forms and who holds it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="20" customHeight="1">
-      <c r="A132" s="22" t="inlineStr">
-        <is>
-          <t>IS STAFF IN UNIFORM?   YES / NO</t>
-        </is>
-      </c>
-      <c r="B132" s="13" t="n"/>
-      <c r="C132" s="13" t="n"/>
-      <c r="D132" s="22" t="inlineStr">
-        <is>
-          <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
-        </is>
-      </c>
-      <c r="E132" s="13" t="n"/>
-      <c r="F132" s="13" t="n"/>
-      <c r="G132" s="13" t="n"/>
-    </row>
-    <row r="133" ht="20" customHeight="1">
-      <c r="A133" s="22" t="inlineStr">
-        <is>
-          <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
-        </is>
-      </c>
-      <c r="B133" s="13" t="n"/>
-      <c r="C133" s="13" t="n"/>
-      <c r="D133" s="22" t="inlineStr">
-        <is>
-          <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
-        </is>
-      </c>
-      <c r="E133" s="13" t="n"/>
-      <c r="F133" s="13" t="n"/>
-      <c r="G133" s="13" t="n"/>
-    </row>
-    <row r="134" ht="20" customHeight="1">
-      <c r="A134" s="22" t="inlineStr">
-        <is>
-          <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
-        </is>
-      </c>
-      <c r="B134" s="13" t="n"/>
-      <c r="C134" s="13" t="n"/>
-      <c r="D134" s="13" t="n"/>
-      <c r="E134" s="13" t="n"/>
-      <c r="F134" s="13" t="n"/>
-      <c r="G134" s="13" t="n"/>
-    </row>
-    <row r="136" ht="18" customHeight="1">
-      <c r="A136" s="6" t="inlineStr">
-        <is>
-          <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
-        </is>
-      </c>
-      <c r="B136" s="7" t="n"/>
-      <c r="C136" s="7" t="n"/>
-      <c r="D136" s="7" t="n"/>
-      <c r="E136" s="7" t="n"/>
-      <c r="F136" s="7" t="n"/>
-      <c r="G136" s="7" t="n"/>
-    </row>
-    <row r="137" ht="32" customHeight="1">
-      <c r="A137" s="8" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B137" s="9" t="inlineStr">
-        <is>
-          <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="32" customHeight="1">
-      <c r="A138" s="8" t="inlineStr">
-        <is>
-          <t>SERVERS</t>
-        </is>
-      </c>
-      <c r="B138" s="9" t="inlineStr">
-        <is>
-          <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="32" customHeight="1">
-      <c r="A139" s="8" t="inlineStr">
-        <is>
-          <t>HOST</t>
-        </is>
-      </c>
-      <c r="B139" s="9" t="inlineStr">
-        <is>
-          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. Card at the door when the room is young; it is far easier there than at the bar. Keep the line off the sidewalk and feed the wait to the bar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="32" customHeight="1">
-      <c r="A140" s="8" t="inlineStr">
-        <is>
-          <t>KITCHEN</t>
-        </is>
-      </c>
-      <c r="B140" s="9" t="inlineStr">
-        <is>
-          <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="32" customHeight="1">
-      <c r="A141" s="8" t="inlineStr">
-        <is>
-          <t>SOCIAL</t>
-        </is>
-      </c>
-      <c r="B141" s="9" t="inlineStr">
-        <is>
-          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="32" customHeight="1">
-      <c r="A142" s="8" t="inlineStr">
-        <is>
-          <t>SUPPORT</t>
-        </is>
-      </c>
-      <c r="B142" s="9" t="inlineStr">
-        <is>
-          <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="6" t="inlineStr">
-        <is>
-          <t>POST-GAME &amp; CLOSE</t>
-        </is>
-      </c>
-      <c r="B144" s="7" t="n"/>
-      <c r="C144" s="7" t="n"/>
-      <c r="D144" s="7" t="n"/>
-      <c r="E144" s="7" t="n"/>
-      <c r="F144" s="7" t="n"/>
-      <c r="G144" s="7" t="n"/>
     </row>
     <row r="145" ht="17" customHeight="1">
       <c r="A145" s="21" t="inlineStr">
@@ -2083,7 +2053,7 @@
       </c>
       <c r="B145" s="9" t="inlineStr">
         <is>
-          <t>All hands on the floor BEFORE the final whistle — not after.</t>
+          <t>Bar par DOUBLED — ice, kegs, backups, garnish, glassware, batch.</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2065,7 @@
       </c>
       <c r="B146" s="9" t="inlineStr">
         <is>
-          <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
+          <t>86 board walked with the kitchen, current and visible.</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2077,7 @@
       </c>
       <c r="B147" s="9" t="inlineStr">
         <is>
-          <t>Every void, comp and discount reconciled to a manager name.</t>
+          <t>TVs, sound and the game feed tested before a single guest sits down.</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2089,7 @@
       </c>
       <c r="B148" s="9" t="inlineStr">
         <is>
-          <t>Every refusal or cut-off logged with what happened and who made the call.</t>
+          <t>ID check covered — door and bar know who is carding, and the light works.</t>
         </is>
       </c>
     </row>
@@ -2131,7 +2101,7 @@
       </c>
       <c r="B149" s="9" t="inlineStr">
         <is>
-          <t>Every station back to original position, original condition.</t>
+          <t>Restrooms stocked and clean before doors.</t>
         </is>
       </c>
     </row>
@@ -2143,114 +2113,357 @@
       </c>
       <c r="B150" s="9" t="inlineStr">
         <is>
+          <t>POS, printers and card processing tested with a live ticket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="17" customHeight="1">
+      <c r="A151" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B151" s="9" t="inlineStr">
+        <is>
+          <t>Cash on hand for a bar that will run cash all night.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="17" customHeight="1">
+      <c r="A152" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B152" s="9" t="inlineStr">
+        <is>
+          <t>Door, patio and line plan — where the wait forms and who holds it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="20" customHeight="1">
+      <c r="A154" s="22" t="inlineStr">
+        <is>
+          <t>IS STAFF IN UNIFORM?   YES / NO</t>
+        </is>
+      </c>
+      <c r="B154" s="13" t="n"/>
+      <c r="C154" s="13" t="n"/>
+      <c r="D154" s="22" t="inlineStr">
+        <is>
+          <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
+        </is>
+      </c>
+      <c r="E154" s="13" t="n"/>
+      <c r="F154" s="13" t="n"/>
+      <c r="G154" s="13" t="n"/>
+    </row>
+    <row r="155" ht="20" customHeight="1">
+      <c r="A155" s="22" t="inlineStr">
+        <is>
+          <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
+        </is>
+      </c>
+      <c r="B155" s="13" t="n"/>
+      <c r="C155" s="13" t="n"/>
+      <c r="D155" s="22" t="inlineStr">
+        <is>
+          <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
+        </is>
+      </c>
+      <c r="E155" s="13" t="n"/>
+      <c r="F155" s="13" t="n"/>
+      <c r="G155" s="13" t="n"/>
+    </row>
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="22" t="inlineStr">
+        <is>
+          <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
+        </is>
+      </c>
+      <c r="B156" s="13" t="n"/>
+      <c r="C156" s="13" t="n"/>
+      <c r="D156" s="13" t="n"/>
+      <c r="E156" s="13" t="n"/>
+      <c r="F156" s="13" t="n"/>
+      <c r="G156" s="13" t="n"/>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="n"/>
+      <c r="C158" s="7" t="n"/>
+      <c r="D158" s="7" t="n"/>
+      <c r="E158" s="7" t="n"/>
+      <c r="F158" s="7" t="n"/>
+      <c r="G158" s="7" t="n"/>
+    </row>
+    <row r="159" ht="32" customHeight="1">
+      <c r="A159" s="8" t="inlineStr">
+        <is>
+          <t>BAR</t>
+        </is>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="32" customHeight="1">
+      <c r="A160" s="8" t="inlineStr">
+        <is>
+          <t>SERVERS</t>
+        </is>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="32" customHeight="1">
+      <c r="A161" s="8" t="inlineStr">
+        <is>
+          <t>HOST</t>
+        </is>
+      </c>
+      <c r="B161" s="9" t="inlineStr">
+        <is>
+          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. Card at the door when the room is young; it is far easier there than at the bar. Keep the line off the sidewalk and feed the wait to the bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="32" customHeight="1">
+      <c r="A162" s="8" t="inlineStr">
+        <is>
+          <t>KITCHEN</t>
+        </is>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="32" customHeight="1">
+      <c r="A163" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL</t>
+        </is>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="32" customHeight="1">
+      <c r="A164" s="8" t="inlineStr">
+        <is>
+          <t>SUPPORT</t>
+        </is>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="18" customHeight="1">
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>POST-GAME &amp; CLOSE</t>
+        </is>
+      </c>
+      <c r="B166" s="7" t="n"/>
+      <c r="C166" s="7" t="n"/>
+      <c r="D166" s="7" t="n"/>
+      <c r="E166" s="7" t="n"/>
+      <c r="F166" s="7" t="n"/>
+      <c r="G166" s="7" t="n"/>
+    </row>
+    <row r="167" ht="17" customHeight="1">
+      <c r="A167" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>All hands on the floor BEFORE the final whistle — not after.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="17" customHeight="1">
+      <c r="A168" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B168" s="9" t="inlineStr">
+        <is>
+          <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="17" customHeight="1">
+      <c r="A169" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B169" s="9" t="inlineStr">
+        <is>
+          <t>Every void, comp and discount reconciled to a manager name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="17" customHeight="1">
+      <c r="A170" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B170" s="9" t="inlineStr">
+        <is>
+          <t>Every refusal or cut-off logged with what happened and who made the call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="17" customHeight="1">
+      <c r="A171" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B171" s="9" t="inlineStr">
+        <is>
+          <t>Every station back to original position, original condition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="17" customHeight="1">
+      <c r="A172" s="21" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B172" s="9" t="inlineStr">
+        <is>
           <t>Shift notes written: what we ran out of, where the wait broke down, what changes next game.</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="4" t="inlineStr">
+    <row r="174">
+      <c r="A174" s="4" t="inlineStr">
         <is>
           <t>MARKETING:</t>
         </is>
       </c>
     </row>
-    <row r="153" ht="18" customHeight="1">
-      <c r="A153" s="16" t="n"/>
-      <c r="B153" s="17" t="n"/>
-      <c r="C153" s="17" t="n"/>
-      <c r="D153" s="17" t="n"/>
-      <c r="E153" s="17" t="n"/>
-      <c r="F153" s="17" t="n"/>
-      <c r="G153" s="17" t="n"/>
-    </row>
-    <row r="154" ht="18" customHeight="1">
-      <c r="A154" s="17" t="n"/>
-      <c r="B154" s="17" t="n"/>
-      <c r="C154" s="17" t="n"/>
-      <c r="D154" s="17" t="n"/>
-      <c r="E154" s="17" t="n"/>
-      <c r="F154" s="17" t="n"/>
-      <c r="G154" s="17" t="n"/>
-    </row>
-    <row r="156" ht="28" customHeight="1">
-      <c r="A156" s="23" t="inlineStr">
+    <row r="175" ht="18" customHeight="1">
+      <c r="A175" s="16" t="n"/>
+      <c r="B175" s="17" t="n"/>
+      <c r="C175" s="17" t="n"/>
+      <c r="D175" s="17" t="n"/>
+      <c r="E175" s="17" t="n"/>
+      <c r="F175" s="17" t="n"/>
+      <c r="G175" s="17" t="n"/>
+    </row>
+    <row r="176" ht="18" customHeight="1">
+      <c r="A176" s="17" t="n"/>
+      <c r="B176" s="17" t="n"/>
+      <c r="C176" s="17" t="n"/>
+      <c r="D176" s="17" t="n"/>
+      <c r="E176" s="17" t="n"/>
+      <c r="F176" s="17" t="n"/>
+      <c r="G176" s="17" t="n"/>
+    </row>
+    <row r="178" ht="28" customHeight="1">
+      <c r="A178" s="23" t="inlineStr">
         <is>
           <t>100% of our standards, 100% of the time, at 100% volume. A full house is not an excuse to run at 80% — it is the reason we hold the line.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="71">
+  <mergeCells count="73">
     <mergeCell ref="C16:E16"/>
-    <mergeCell ref="B117:G117"/>
     <mergeCell ref="A14:G14"/>
-    <mergeCell ref="B120:G120"/>
     <mergeCell ref="B145:G145"/>
+    <mergeCell ref="B151:G151"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A133:C133"/>
-    <mergeCell ref="A144:G144"/>
     <mergeCell ref="A22:G22"/>
+    <mergeCell ref="B170:G170"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="B148:G148"/>
     <mergeCell ref="A156:G156"/>
-    <mergeCell ref="A153:G154"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="B119:G119"/>
-    <mergeCell ref="A134:G134"/>
+    <mergeCell ref="A154:C154"/>
+    <mergeCell ref="B171:G171"/>
     <mergeCell ref="D51:G51"/>
     <mergeCell ref="A19:G19"/>
-    <mergeCell ref="B116:G116"/>
-    <mergeCell ref="D133:G133"/>
     <mergeCell ref="B147:G147"/>
+    <mergeCell ref="B162:G162"/>
     <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A115:G115"/>
+    <mergeCell ref="A93:G93"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="D132:G132"/>
-    <mergeCell ref="B137:G137"/>
+    <mergeCell ref="B172:G172"/>
+    <mergeCell ref="B168:G168"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C10:G10"/>
-    <mergeCell ref="B128:G128"/>
     <mergeCell ref="B146:G146"/>
-    <mergeCell ref="B118:G118"/>
     <mergeCell ref="A92:G92"/>
-    <mergeCell ref="B127:G127"/>
     <mergeCell ref="A15:G15"/>
+    <mergeCell ref="B143:G143"/>
+    <mergeCell ref="A166:G166"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="B139:G139"/>
-    <mergeCell ref="B124:G124"/>
+    <mergeCell ref="A178:G178"/>
     <mergeCell ref="B142:G142"/>
+    <mergeCell ref="D155:G155"/>
+    <mergeCell ref="B164:G164"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B123:G123"/>
+    <mergeCell ref="A134:G135"/>
+    <mergeCell ref="A155:C155"/>
+    <mergeCell ref="A158:G158"/>
+    <mergeCell ref="B160:G160"/>
+    <mergeCell ref="B169:G169"/>
+    <mergeCell ref="A175:G176"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="A47:G48"/>
-    <mergeCell ref="B126:G126"/>
+    <mergeCell ref="B163:G163"/>
+    <mergeCell ref="B144:G144"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A112:G113"/>
     <mergeCell ref="B138:G138"/>
-    <mergeCell ref="B129:G129"/>
+    <mergeCell ref="A137:G137"/>
     <mergeCell ref="A35:G36"/>
-    <mergeCell ref="B125:G125"/>
+    <mergeCell ref="D154:G154"/>
     <mergeCell ref="A74:G74"/>
-    <mergeCell ref="B121:G121"/>
+    <mergeCell ref="B141:G141"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A56:G56"/>
     <mergeCell ref="D53:G53"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A43:G44"/>
-    <mergeCell ref="B122:G122"/>
+    <mergeCell ref="B150:G150"/>
     <mergeCell ref="A50:G50"/>
     <mergeCell ref="A39:G40"/>
-    <mergeCell ref="A132:C132"/>
+    <mergeCell ref="B140:G140"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A136:G136"/>
+    <mergeCell ref="B149:G149"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B140:G140"/>
-    <mergeCell ref="B149:G149"/>
-    <mergeCell ref="B150:G150"/>
-    <mergeCell ref="B130:G130"/>
-    <mergeCell ref="B141:G141"/>
+    <mergeCell ref="B159:G159"/>
+    <mergeCell ref="B167:G167"/>
+    <mergeCell ref="A113:G113"/>
+    <mergeCell ref="B161:G161"/>
+    <mergeCell ref="B152:G152"/>
     <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rename host lead to first in command and add a second
Host stations now read: first in command, second in command, runner, waters,
bathrooms — in both the AM and PM blocks. The host position brief says second
steps in the moment first gets pulled, so the door never goes unowned.

Widened column A in the workbook so the longer labels clear their write lines.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -558,7 +558,7 @@
   <dimension ref="A1:G178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16.5" customWidth="1" min="1" max="1"/>
+    <col width="20.5" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -1542,7 +1542,7 @@
     <row r="95" ht="18" customHeight="1">
       <c r="A95" s="20" t="inlineStr">
         <is>
-          <t>Lead:</t>
+          <t>First in command:</t>
         </is>
       </c>
       <c r="B95" s="5" t="n"/>
@@ -1563,7 +1563,7 @@
     <row r="96" ht="18" customHeight="1">
       <c r="A96" s="20" t="inlineStr">
         <is>
-          <t>Runner:</t>
+          <t>Second in command:</t>
         </is>
       </c>
       <c r="B96" s="5" t="n"/>
@@ -1584,7 +1584,7 @@
     <row r="97" ht="18" customHeight="1">
       <c r="A97" s="20" t="inlineStr">
         <is>
-          <t>Waters:</t>
+          <t>Runner:</t>
         </is>
       </c>
       <c r="B97" s="5" t="n"/>
@@ -1605,7 +1605,7 @@
     <row r="98" ht="18" customHeight="1">
       <c r="A98" s="20" t="inlineStr">
         <is>
-          <t>Bathrooms:</t>
+          <t>Waters:</t>
         </is>
       </c>
       <c r="B98" s="5" t="n"/>
@@ -1618,6 +1618,12 @@
       <c r="G98" s="5" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="20" t="inlineStr">
+        <is>
+          <t>Bathrooms:</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="n"/>
       <c r="E99" s="20" t="inlineStr">
         <is>
           <t>Patio:</t>
@@ -1746,7 +1752,7 @@
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="20" t="inlineStr">
         <is>
-          <t>Lead:</t>
+          <t>First in command:</t>
         </is>
       </c>
       <c r="B115" s="5" t="n"/>
@@ -1767,7 +1773,7 @@
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="20" t="inlineStr">
         <is>
-          <t>Runner:</t>
+          <t>Second in command:</t>
         </is>
       </c>
       <c r="B116" s="5" t="n"/>
@@ -1788,7 +1794,7 @@
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="20" t="inlineStr">
         <is>
-          <t>Waters:</t>
+          <t>Runner:</t>
         </is>
       </c>
       <c r="B117" s="5" t="n"/>
@@ -1809,7 +1815,7 @@
     <row r="118" ht="18" customHeight="1">
       <c r="A118" s="20" t="inlineStr">
         <is>
-          <t>Bathrooms:</t>
+          <t>Waters:</t>
         </is>
       </c>
       <c r="B118" s="5" t="n"/>
@@ -1822,6 +1828,12 @@
       <c r="G118" s="5" t="n"/>
     </row>
     <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="20" t="inlineStr">
+        <is>
+          <t>Bathrooms:</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="n"/>
       <c r="E119" s="20" t="inlineStr">
         <is>
           <t>Patio:</t>
@@ -2233,7 +2245,7 @@
       </c>
       <c r="B161" s="9" t="inlineStr">
         <is>
-          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. Card at the door when the room is young; it is far easier there than at the bar. Keep the line off the sidewalk and feed the wait to the bar.</t>
+          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. First in command runs the book; second in command steps in the moment first gets pulled. Card at the door when the room is young. Keep the line off the sidewalk and feed the wait to the bar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a trainee count to every staff count line
Staff #'s now carries two numbers per role — ON and IN TRAINING — for all
eight roles, in both the AM and PM blocks, so a manager can see at a glance
how much of the crew is still learning the station.

Staff to coach and 7shifts completion move to their own row underneath to
make room for the second column.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -1097,14 +1097,19 @@
           <t>STAFF #'S</t>
         </is>
       </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
+          <t>IN TRAINING</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
           <t>SHIFT LEADS</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>STAFF TO COACH — 1 HUDDL</t>
         </is>
       </c>
     </row>
@@ -1115,11 +1120,7 @@
         </is>
       </c>
       <c r="B58" s="5" t="n"/>
-      <c r="C58" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
+      <c r="C58" s="5" t="n"/>
       <c r="D58" s="5" t="n"/>
       <c r="E58" s="20" t="inlineStr">
         <is>
@@ -1136,15 +1137,11 @@
         </is>
       </c>
       <c r="B59" s="5" t="n"/>
-      <c r="C59" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
+      <c r="C59" s="5" t="n"/>
       <c r="D59" s="5" t="n"/>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>BAR:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="F59" s="5" t="n"/>
@@ -1157,15 +1154,11 @@
         </is>
       </c>
       <c r="B60" s="5" t="n"/>
-      <c r="C60" s="20" t="inlineStr">
-        <is>
-          <t>BARTENDER:</t>
-        </is>
-      </c>
+      <c r="C60" s="5" t="n"/>
       <c r="D60" s="5" t="n"/>
       <c r="E60" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>BARTENDER:</t>
         </is>
       </c>
       <c r="F60" s="5" t="n"/>
@@ -1178,11 +1171,7 @@
         </is>
       </c>
       <c r="B61" s="5" t="n"/>
-      <c r="C61" s="20" t="inlineStr">
-        <is>
-          <t>HOST:</t>
-        </is>
-      </c>
+      <c r="C61" s="5" t="n"/>
       <c r="D61" s="5" t="n"/>
       <c r="E61" s="20" t="inlineStr">
         <is>
@@ -1199,15 +1188,11 @@
         </is>
       </c>
       <c r="B62" s="5" t="n"/>
-      <c r="C62" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
+      <c r="C62" s="5" t="n"/>
       <c r="D62" s="5" t="n"/>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>BARBACK:</t>
+          <t>BAR:</t>
         </is>
       </c>
       <c r="F62" s="5" t="n"/>
@@ -1220,12 +1205,15 @@
         </is>
       </c>
       <c r="B63" s="5" t="n"/>
-      <c r="C63" s="20" t="inlineStr">
+      <c r="C63" s="5" t="n"/>
+      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="20" t="inlineStr">
         <is>
           <t>BARBACK:</t>
         </is>
       </c>
-      <c r="D63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
+      <c r="G63" s="5" t="n"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="20" t="inlineStr">
@@ -1234,6 +1222,8 @@
         </is>
       </c>
       <c r="B64" s="5" t="n"/>
+      <c r="C64" s="5" t="n"/>
+      <c r="D64" s="5" t="n"/>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="20" t="inlineStr">
@@ -1242,10 +1232,17 @@
         </is>
       </c>
       <c r="B65" s="5" t="n"/>
+      <c r="C65" s="5" t="n"/>
+      <c r="D65" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
+          <t>STAFF TO COACH — 1 HUDDL</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
           <t>7SHIFTS COMPLETION</t>
         </is>
       </c>
@@ -1257,6 +1254,12 @@
         </is>
       </c>
       <c r="B68" s="5" t="n"/>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="n"/>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="20" t="inlineStr">
@@ -1265,6 +1268,12 @@
         </is>
       </c>
       <c r="B69" s="5" t="n"/>
+      <c r="C69" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="n"/>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="20" t="inlineStr">
@@ -1273,6 +1282,12 @@
         </is>
       </c>
       <c r="B70" s="5" t="n"/>
+      <c r="C70" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="20" t="inlineStr">
@@ -1281,6 +1296,12 @@
         </is>
       </c>
       <c r="B71" s="5" t="n"/>
+      <c r="C71" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="n"/>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="20" t="inlineStr">
@@ -1289,6 +1310,12 @@
         </is>
       </c>
       <c r="B72" s="5" t="n"/>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="n"/>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
@@ -1309,14 +1336,19 @@
           <t>STAFF #'S</t>
         </is>
       </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
+          <t>IN TRAINING</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
           <t>SHIFT LEADS</t>
-        </is>
-      </c>
-      <c r="E75" s="8" t="inlineStr">
-        <is>
-          <t>STAFF TO COACH — 1 HUDDL</t>
         </is>
       </c>
     </row>
@@ -1327,11 +1359,7 @@
         </is>
       </c>
       <c r="B76" s="5" t="n"/>
-      <c r="C76" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
+      <c r="C76" s="5" t="n"/>
       <c r="D76" s="5" t="n"/>
       <c r="E76" s="20" t="inlineStr">
         <is>
@@ -1348,15 +1376,11 @@
         </is>
       </c>
       <c r="B77" s="5" t="n"/>
-      <c r="C77" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
+      <c r="C77" s="5" t="n"/>
       <c r="D77" s="5" t="n"/>
       <c r="E77" s="20" t="inlineStr">
         <is>
-          <t>BAR:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="F77" s="5" t="n"/>
@@ -1369,15 +1393,11 @@
         </is>
       </c>
       <c r="B78" s="5" t="n"/>
-      <c r="C78" s="20" t="inlineStr">
-        <is>
-          <t>BARTENDER:</t>
-        </is>
-      </c>
+      <c r="C78" s="5" t="n"/>
       <c r="D78" s="5" t="n"/>
       <c r="E78" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>BARTENDER:</t>
         </is>
       </c>
       <c r="F78" s="5" t="n"/>
@@ -1390,11 +1410,7 @@
         </is>
       </c>
       <c r="B79" s="5" t="n"/>
-      <c r="C79" s="20" t="inlineStr">
-        <is>
-          <t>HOST:</t>
-        </is>
-      </c>
+      <c r="C79" s="5" t="n"/>
       <c r="D79" s="5" t="n"/>
       <c r="E79" s="20" t="inlineStr">
         <is>
@@ -1411,15 +1427,11 @@
         </is>
       </c>
       <c r="B80" s="5" t="n"/>
-      <c r="C80" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
+      <c r="C80" s="5" t="n"/>
       <c r="D80" s="5" t="n"/>
       <c r="E80" s="20" t="inlineStr">
         <is>
-          <t>BARBACK:</t>
+          <t>BAR:</t>
         </is>
       </c>
       <c r="F80" s="5" t="n"/>
@@ -1432,12 +1444,15 @@
         </is>
       </c>
       <c r="B81" s="5" t="n"/>
-      <c r="C81" s="20" t="inlineStr">
+      <c r="C81" s="5" t="n"/>
+      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="20" t="inlineStr">
         <is>
           <t>BARBACK:</t>
         </is>
       </c>
-      <c r="D81" s="5" t="n"/>
+      <c r="F81" s="5" t="n"/>
+      <c r="G81" s="5" t="n"/>
     </row>
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="20" t="inlineStr">
@@ -1446,6 +1461,8 @@
         </is>
       </c>
       <c r="B82" s="5" t="n"/>
+      <c r="C82" s="5" t="n"/>
+      <c r="D82" s="5" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="20" t="inlineStr">
@@ -1454,10 +1471,17 @@
         </is>
       </c>
       <c r="B83" s="5" t="n"/>
+      <c r="C83" s="5" t="n"/>
+      <c r="D83" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
+          <t>STAFF TO COACH — 1 HUDDL</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
           <t>7SHIFTS COMPLETION</t>
         </is>
       </c>
@@ -1469,6 +1493,12 @@
         </is>
       </c>
       <c r="B86" s="5" t="n"/>
+      <c r="C86" s="20" t="inlineStr">
+        <is>
+          <t>SERVER:</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="n"/>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="20" t="inlineStr">
@@ -1477,6 +1507,12 @@
         </is>
       </c>
       <c r="B87" s="5" t="n"/>
+      <c r="C87" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="n"/>
     </row>
     <row r="88" ht="18" customHeight="1">
       <c r="A88" s="20" t="inlineStr">
@@ -1485,6 +1521,12 @@
         </is>
       </c>
       <c r="B88" s="5" t="n"/>
+      <c r="C88" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="n"/>
     </row>
     <row r="89" ht="18" customHeight="1">
       <c r="A89" s="20" t="inlineStr">
@@ -1493,6 +1535,12 @@
         </is>
       </c>
       <c r="B89" s="5" t="n"/>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="20" t="inlineStr">
@@ -1501,6 +1549,12 @@
         </is>
       </c>
       <c r="B90" s="5" t="n"/>
+      <c r="C90" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1">
       <c r="A92" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Total the staff counts for each crew
Each crew's staff block now ends in two calculated rows: TOTAL SCHEDULED
(sums the scheduled and in-training columns) and TOTAL STAFF ON SHIFT
(scheduled + in training).

The workbook uses real SUM formulas over the eight role rows, so it
recalculates as the counts are typed. The web version totals the same three
numbers live as you fill it in.

No AM+PM day total: staff who work both shifts would be counted twice.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Game Day Pre-Shift" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$178</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -104,7 +104,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -127,11 +127,14 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <top style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,6 +182,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -555,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G178"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.5" customWidth="1" min="1" max="1"/>
@@ -1235,56 +1245,60 @@
       <c r="C65" s="5" t="n"/>
       <c r="D65" s="5" t="n"/>
     </row>
-    <row r="67">
+    <row r="66" ht="19" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL SCHEDULED:</t>
+        </is>
+      </c>
+      <c r="B66" s="21">
+        <f>SUM(B58:B65)</f>
+        <v/>
+      </c>
+      <c r="C66" s="21">
+        <f>SUM(C58:C65)</f>
+        <v/>
+      </c>
+      <c r="D66" s="22" t="n"/>
+    </row>
+    <row r="67" ht="19" customHeight="1">
       <c r="A67" s="8" t="inlineStr">
         <is>
+          <t>TOTAL STAFF ON SHIFT:</t>
+        </is>
+      </c>
+      <c r="B67" s="4">
+        <f>B66+C66</f>
+        <v/>
+      </c>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>(scheduled + in training)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
           <t>STAFF TO COACH — 1 HUDDL</t>
         </is>
       </c>
-      <c r="C67" s="8" t="inlineStr">
+      <c r="C69" s="8" t="inlineStr">
         <is>
           <t>7SHIFTS COMPLETION</t>
         </is>
       </c>
-    </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="n"/>
-      <c r="C68" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="n"/>
-    </row>
-    <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="n"/>
-      <c r="C69" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="n"/>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="B70" s="5" t="n"/>
       <c r="C70" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="D70" s="5" t="n"/>
@@ -1292,13 +1306,13 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="20" t="inlineStr">
         <is>
-          <t>HOST:</t>
+          <t>BAR:</t>
         </is>
       </c>
       <c r="B71" s="5" t="n"/>
       <c r="C71" s="20" t="inlineStr">
         <is>
-          <t>HOST:</t>
+          <t>BAR:</t>
         </is>
       </c>
       <c r="D71" s="5" t="n"/>
@@ -1306,90 +1320,84 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="20" t="inlineStr">
         <is>
-          <t>BARBACK:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="B72" s="5" t="n"/>
       <c r="C72" s="20" t="inlineStr">
         <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="n"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n"/>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="n"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="20" t="inlineStr">
+        <is>
           <t>BARBACK:</t>
         </is>
       </c>
-      <c r="D72" s="5" t="n"/>
-    </row>
-    <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="n"/>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>PM CREW — STAFF #'S &amp; COMPLETIONS</t>
         </is>
       </c>
-      <c r="B74" s="7" t="n"/>
-      <c r="C74" s="7" t="n"/>
-      <c r="D74" s="7" t="n"/>
-      <c r="E74" s="7" t="n"/>
-      <c r="F74" s="7" t="n"/>
-      <c r="G74" s="7" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="B76" s="7" t="n"/>
+      <c r="C76" s="7" t="n"/>
+      <c r="D76" s="7" t="n"/>
+      <c r="E76" s="7" t="n"/>
+      <c r="F76" s="7" t="n"/>
+      <c r="G76" s="7" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
         <is>
           <t>STAFF #'S</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B77" s="8" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="C75" s="8" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t>IN TRAINING</t>
         </is>
       </c>
-      <c r="E75" s="8" t="inlineStr">
+      <c r="E77" s="8" t="inlineStr">
         <is>
           <t>SHIFT LEADS</t>
         </is>
       </c>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="20" t="inlineStr">
-        <is>
-          <t>SERVERS:</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="n"/>
-      <c r="C76" s="5" t="n"/>
-      <c r="D76" s="5" t="n"/>
-      <c r="E76" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="F76" s="5" t="n"/>
-      <c r="G76" s="5" t="n"/>
-    </row>
-    <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="20" t="inlineStr">
-        <is>
-          <t>BARTENDERS:</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="n"/>
-      <c r="C77" s="5" t="n"/>
-      <c r="D77" s="5" t="n"/>
-      <c r="E77" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
-      <c r="F77" s="5" t="n"/>
-      <c r="G77" s="5" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="20" t="inlineStr">
         <is>
-          <t>CAFÉ:</t>
+          <t>SERVERS:</t>
         </is>
       </c>
       <c r="B78" s="5" t="n"/>
@@ -1397,7 +1405,7 @@
       <c r="D78" s="5" t="n"/>
       <c r="E78" s="20" t="inlineStr">
         <is>
-          <t>BARTENDER:</t>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="F78" s="5" t="n"/>
@@ -1406,7 +1414,7 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="20" t="inlineStr">
         <is>
-          <t>HOSTS:</t>
+          <t>BARTENDERS:</t>
         </is>
       </c>
       <c r="B79" s="5" t="n"/>
@@ -1414,7 +1422,7 @@
       <c r="D79" s="5" t="n"/>
       <c r="E79" s="20" t="inlineStr">
         <is>
-          <t>HOST:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="F79" s="5" t="n"/>
@@ -1423,7 +1431,7 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="20" t="inlineStr">
         <is>
-          <t>RUNNERS:</t>
+          <t>CAFÉ:</t>
         </is>
       </c>
       <c r="B80" s="5" t="n"/>
@@ -1431,7 +1439,7 @@
       <c r="D80" s="5" t="n"/>
       <c r="E80" s="20" t="inlineStr">
         <is>
-          <t>BAR:</t>
+          <t>BARTENDER:</t>
         </is>
       </c>
       <c r="F80" s="5" t="n"/>
@@ -1440,7 +1448,7 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="20" t="inlineStr">
         <is>
-          <t>BARBACKS:</t>
+          <t>HOSTS:</t>
         </is>
       </c>
       <c r="B81" s="5" t="n"/>
@@ -1448,7 +1456,7 @@
       <c r="D81" s="5" t="n"/>
       <c r="E81" s="20" t="inlineStr">
         <is>
-          <t>BARBACK:</t>
+          <t>HOST:</t>
         </is>
       </c>
       <c r="F81" s="5" t="n"/>
@@ -1457,268 +1465,281 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="20" t="inlineStr">
         <is>
-          <t>SHOT GIRL:</t>
+          <t>RUNNERS:</t>
         </is>
       </c>
       <c r="B82" s="5" t="n"/>
       <c r="C82" s="5" t="n"/>
       <c r="D82" s="5" t="n"/>
+      <c r="E82" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="n"/>
+      <c r="G82" s="5" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="20" t="inlineStr">
         <is>
-          <t>MANAGERS:</t>
+          <t>BARBACKS:</t>
         </is>
       </c>
       <c r="B83" s="5" t="n"/>
       <c r="C83" s="5" t="n"/>
       <c r="D83" s="5" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="8" t="inlineStr">
+      <c r="E83" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="n"/>
+      <c r="G83" s="5" t="n"/>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="20" t="inlineStr">
+        <is>
+          <t>SHOT GIRL:</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n"/>
+      <c r="C84" s="5" t="n"/>
+      <c r="D84" s="5" t="n"/>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="20" t="inlineStr">
+        <is>
+          <t>MANAGERS:</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="n"/>
+      <c r="C85" s="5" t="n"/>
+      <c r="D85" s="5" t="n"/>
+    </row>
+    <row r="86" ht="19" customHeight="1">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL SCHEDULED:</t>
+        </is>
+      </c>
+      <c r="B86" s="21">
+        <f>SUM(B78:B85)</f>
+        <v/>
+      </c>
+      <c r="C86" s="21">
+        <f>SUM(C78:C85)</f>
+        <v/>
+      </c>
+      <c r="D86" s="22" t="n"/>
+    </row>
+    <row r="87" ht="19" customHeight="1">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL STAFF ON SHIFT:</t>
+        </is>
+      </c>
+      <c r="B87" s="4">
+        <f>B86+C86</f>
+        <v/>
+      </c>
+      <c r="C87" s="23" t="inlineStr">
+        <is>
+          <t>(scheduled + in training)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
         <is>
           <t>STAFF TO COACH — 1 HUDDL</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr">
         <is>
           <t>7SHIFTS COMPLETION</t>
         </is>
       </c>
-    </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="n"/>
-      <c r="C86" s="20" t="inlineStr">
-        <is>
-          <t>SERVER:</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="n"/>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="n"/>
-      <c r="C87" s="20" t="inlineStr">
-        <is>
-          <t>BAR:</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="n"/>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
-      <c r="B88" s="5" t="n"/>
-      <c r="C88" s="20" t="inlineStr">
-        <is>
-          <t>CAFÉ:</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="n"/>
-    </row>
-    <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="20" t="inlineStr">
-        <is>
-          <t>HOST:</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="n"/>
-      <c r="C89" s="20" t="inlineStr">
-        <is>
-          <t>HOST:</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="n"/>
     </row>
     <row r="90" ht="18" customHeight="1">
       <c r="A90" s="20" t="inlineStr">
         <is>
-          <t>BARBACK:</t>
+          <t>SERVER:</t>
         </is>
       </c>
       <c r="B90" s="5" t="n"/>
       <c r="C90" s="20" t="inlineStr">
         <is>
+          <t>SERVER:</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="n"/>
+      <c r="C91" s="20" t="inlineStr">
+        <is>
+          <t>BAR:</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="n"/>
+      <c r="C92" s="20" t="inlineStr">
+        <is>
+          <t>CAFÉ:</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="n"/>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t>HOST:</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="20" t="inlineStr">
+        <is>
           <t>BARBACK:</t>
         </is>
       </c>
-      <c r="D90" s="5" t="n"/>
-    </row>
-    <row r="92" ht="18" customHeight="1">
-      <c r="A92" s="6" t="inlineStr">
+      <c r="B94" s="5" t="n"/>
+      <c r="C94" s="20" t="inlineStr">
+        <is>
+          <t>BARBACK:</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>STATION ASSIGNMENTS — WRITE A NAME ON EVERY LINE</t>
         </is>
       </c>
-      <c r="B92" s="7" t="n"/>
-      <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="n"/>
-      <c r="E92" s="7" t="n"/>
-      <c r="F92" s="7" t="n"/>
-      <c r="G92" s="7" t="n"/>
-    </row>
-    <row r="93" ht="17" customHeight="1">
-      <c r="A93" s="8" t="inlineStr">
+      <c r="B96" s="7" t="n"/>
+      <c r="C96" s="7" t="n"/>
+      <c r="D96" s="7" t="n"/>
+      <c r="E96" s="7" t="n"/>
+      <c r="F96" s="7" t="n"/>
+      <c r="G96" s="7" t="n"/>
+    </row>
+    <row r="97" ht="17" customHeight="1">
+      <c r="A97" s="8" t="inlineStr">
         <is>
           <t>AM CREW</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
         <is>
           <t>HOST</t>
         </is>
       </c>
-      <c r="C94" s="8" t="inlineStr">
+      <c r="C98" s="8" t="inlineStr">
         <is>
           <t>RUNNERS</t>
         </is>
       </c>
-      <c r="E94" s="8" t="inlineStr">
+      <c r="E98" s="8" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="20" t="inlineStr">
-        <is>
-          <t>First in command:</t>
-        </is>
-      </c>
-      <c r="B95" s="5" t="n"/>
-      <c r="C95" s="20" t="inlineStr">
-        <is>
-          <t>Bar 100:</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="n"/>
-      <c r="E95" s="20" t="inlineStr">
-        <is>
-          <t>100:</t>
-        </is>
-      </c>
-      <c r="F95" s="5" t="n"/>
-      <c r="G95" s="5" t="n"/>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="20" t="inlineStr">
-        <is>
-          <t>Second in command:</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="n"/>
-      <c r="C96" s="20" t="inlineStr">
-        <is>
-          <t>Bar 200:</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="n"/>
-      <c r="E96" s="20" t="inlineStr">
-        <is>
-          <t>105:</t>
-        </is>
-      </c>
-      <c r="F96" s="5" t="n"/>
-      <c r="G96" s="5" t="n"/>
-    </row>
-    <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="20" t="inlineStr">
-        <is>
-          <t>Runner:</t>
-        </is>
-      </c>
-      <c r="B97" s="5" t="n"/>
-      <c r="C97" s="20" t="inlineStr">
-        <is>
-          <t>Food:</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="n"/>
-      <c r="E97" s="20" t="inlineStr">
-        <is>
-          <t>110:</t>
-        </is>
-      </c>
-      <c r="F97" s="5" t="n"/>
-      <c r="G97" s="5" t="n"/>
-    </row>
-    <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="20" t="inlineStr">
-        <is>
-          <t>Waters:</t>
-        </is>
-      </c>
-      <c r="B98" s="5" t="n"/>
-      <c r="E98" s="20" t="inlineStr">
-        <is>
-          <t>200:</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="n"/>
-      <c r="G98" s="5" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="20" t="inlineStr">
         <is>
-          <t>Bathrooms:</t>
+          <t>First in command:</t>
         </is>
       </c>
       <c r="B99" s="5" t="n"/>
+      <c r="C99" s="20" t="inlineStr">
+        <is>
+          <t>Bar 100:</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="n"/>
       <c r="E99" s="20" t="inlineStr">
         <is>
-          <t>Patio:</t>
+          <t>100:</t>
         </is>
       </c>
       <c r="F99" s="5" t="n"/>
       <c r="G99" s="5" t="n"/>
     </row>
-    <row r="101">
-      <c r="A101" s="8" t="inlineStr">
-        <is>
-          <t>BARBACKS</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t>SHOT GIRL</t>
-        </is>
-      </c>
-      <c r="E101" s="8" t="inlineStr">
-        <is>
-          <t>TASTE PLATE</t>
-        </is>
-      </c>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="20" t="inlineStr">
+        <is>
+          <t>Second in command:</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="n"/>
+      <c r="C100" s="20" t="inlineStr">
+        <is>
+          <t>Bar 200:</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="n"/>
+      <c r="E100" s="20" t="inlineStr">
+        <is>
+          <t>105:</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="n"/>
+      <c r="G100" s="5" t="n"/>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="20" t="inlineStr">
+        <is>
+          <t>Runner:</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="n"/>
+      <c r="C101" s="20" t="inlineStr">
+        <is>
+          <t>Food:</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="n"/>
+      <c r="E101" s="20" t="inlineStr">
+        <is>
+          <t>110:</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="n"/>
+      <c r="G101" s="5" t="n"/>
     </row>
     <row r="102" ht="18" customHeight="1">
       <c r="A102" s="20" t="inlineStr">
         <is>
-          <t>Main Bar:</t>
+          <t>Waters:</t>
         </is>
       </c>
       <c r="B102" s="5" t="n"/>
-      <c r="C102" s="20" t="inlineStr">
-        <is>
-          <t>On tonight:</t>
-        </is>
-      </c>
-      <c r="D102" s="5" t="n"/>
       <c r="E102" s="20" t="inlineStr">
         <is>
-          <t>Running it:</t>
+          <t>200:</t>
         </is>
       </c>
       <c r="F102" s="5" t="n"/>
@@ -1727,46 +1748,76 @@
     <row r="103" ht="18" customHeight="1">
       <c r="A103" s="20" t="inlineStr">
         <is>
-          <t>Patio Bar:</t>
+          <t>Bathrooms:</t>
         </is>
       </c>
       <c r="B103" s="5" t="n"/>
-    </row>
-    <row r="104" ht="18" customHeight="1">
-      <c r="A104" s="20" t="inlineStr">
-        <is>
-          <t>Main Floor:</t>
-        </is>
-      </c>
-      <c r="B104" s="5" t="n"/>
-    </row>
-    <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="20" t="inlineStr">
-        <is>
-          <t>Café:</t>
-        </is>
-      </c>
-      <c r="B105" s="5" t="n"/>
+      <c r="E103" s="20" t="inlineStr">
+        <is>
+          <t>Patio:</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="n"/>
+      <c r="G103" s="5" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>BARBACKS</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>SHOT GIRL</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>TASTE PLATE</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="20" t="inlineStr">
         <is>
-          <t>Front Patio:</t>
+          <t>Main Bar:</t>
         </is>
       </c>
       <c r="B106" s="5" t="n"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="8" t="inlineStr">
-        <is>
-          <t>SOCIAL MEDIA</t>
-        </is>
-      </c>
+      <c r="C106" s="20" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="D106" s="5" t="n"/>
+      <c r="E106" s="20" t="inlineStr">
+        <is>
+          <t>Running it:</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="n"/>
+      <c r="G106" s="5" t="n"/>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="20" t="inlineStr">
+        <is>
+          <t>Patio Bar:</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="n"/>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="20" t="inlineStr">
+        <is>
+          <t>Main Floor:</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="n"/>
     </row>
     <row r="109" ht="18" customHeight="1">
       <c r="A109" s="20" t="inlineStr">
         <is>
-          <t>On tonight:</t>
+          <t>Café:</t>
         </is>
       </c>
       <c r="B109" s="5" t="n"/>
@@ -1774,161 +1825,131 @@
     <row r="110" ht="18" customHeight="1">
       <c r="A110" s="20" t="inlineStr">
         <is>
+          <t>Front Patio:</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL MEDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="20" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="n"/>
+    </row>
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="20" t="inlineStr">
+        <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B110" s="5" t="n"/>
-    </row>
-    <row r="113" ht="17" customHeight="1">
-      <c r="A113" s="8" t="inlineStr">
+      <c r="B114" s="5" t="n"/>
+    </row>
+    <row r="117" ht="17" customHeight="1">
+      <c r="A117" s="8" t="inlineStr">
         <is>
           <t>PM CREW</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="8" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
         <is>
           <t>HOST</t>
         </is>
       </c>
-      <c r="C114" s="8" t="inlineStr">
+      <c r="C118" s="8" t="inlineStr">
         <is>
           <t>RUNNERS</t>
         </is>
       </c>
-      <c r="E114" s="8" t="inlineStr">
+      <c r="E118" s="8" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
-    </row>
-    <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="20" t="inlineStr">
-        <is>
-          <t>First in command:</t>
-        </is>
-      </c>
-      <c r="B115" s="5" t="n"/>
-      <c r="C115" s="20" t="inlineStr">
-        <is>
-          <t>Bar 100:</t>
-        </is>
-      </c>
-      <c r="D115" s="5" t="n"/>
-      <c r="E115" s="20" t="inlineStr">
-        <is>
-          <t>100:</t>
-        </is>
-      </c>
-      <c r="F115" s="5" t="n"/>
-      <c r="G115" s="5" t="n"/>
-    </row>
-    <row r="116" ht="18" customHeight="1">
-      <c r="A116" s="20" t="inlineStr">
-        <is>
-          <t>Second in command:</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="n"/>
-      <c r="C116" s="20" t="inlineStr">
-        <is>
-          <t>Bar 200:</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="n"/>
-      <c r="E116" s="20" t="inlineStr">
-        <is>
-          <t>105:</t>
-        </is>
-      </c>
-      <c r="F116" s="5" t="n"/>
-      <c r="G116" s="5" t="n"/>
-    </row>
-    <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="20" t="inlineStr">
-        <is>
-          <t>Runner:</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="n"/>
-      <c r="C117" s="20" t="inlineStr">
-        <is>
-          <t>Food:</t>
-        </is>
-      </c>
-      <c r="D117" s="5" t="n"/>
-      <c r="E117" s="20" t="inlineStr">
-        <is>
-          <t>110:</t>
-        </is>
-      </c>
-      <c r="F117" s="5" t="n"/>
-      <c r="G117" s="5" t="n"/>
-    </row>
-    <row r="118" ht="18" customHeight="1">
-      <c r="A118" s="20" t="inlineStr">
-        <is>
-          <t>Waters:</t>
-        </is>
-      </c>
-      <c r="B118" s="5" t="n"/>
-      <c r="E118" s="20" t="inlineStr">
-        <is>
-          <t>200:</t>
-        </is>
-      </c>
-      <c r="F118" s="5" t="n"/>
-      <c r="G118" s="5" t="n"/>
     </row>
     <row r="119" ht="18" customHeight="1">
       <c r="A119" s="20" t="inlineStr">
         <is>
-          <t>Bathrooms:</t>
+          <t>First in command:</t>
         </is>
       </c>
       <c r="B119" s="5" t="n"/>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>Bar 100:</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="n"/>
       <c r="E119" s="20" t="inlineStr">
         <is>
-          <t>Patio:</t>
+          <t>100:</t>
         </is>
       </c>
       <c r="F119" s="5" t="n"/>
       <c r="G119" s="5" t="n"/>
     </row>
-    <row r="121">
-      <c r="A121" s="8" t="inlineStr">
-        <is>
-          <t>BARBACKS</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="inlineStr">
-        <is>
-          <t>SHOT GIRL</t>
-        </is>
-      </c>
-      <c r="E121" s="8" t="inlineStr">
-        <is>
-          <t>TASTE PLATE</t>
-        </is>
-      </c>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="20" t="inlineStr">
+        <is>
+          <t>Second in command:</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="n"/>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t>Bar 200:</t>
+        </is>
+      </c>
+      <c r="D120" s="5" t="n"/>
+      <c r="E120" s="20" t="inlineStr">
+        <is>
+          <t>105:</t>
+        </is>
+      </c>
+      <c r="F120" s="5" t="n"/>
+      <c r="G120" s="5" t="n"/>
+    </row>
+    <row r="121" ht="18" customHeight="1">
+      <c r="A121" s="20" t="inlineStr">
+        <is>
+          <t>Runner:</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="n"/>
+      <c r="C121" s="20" t="inlineStr">
+        <is>
+          <t>Food:</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="n"/>
+      <c r="E121" s="20" t="inlineStr">
+        <is>
+          <t>110:</t>
+        </is>
+      </c>
+      <c r="F121" s="5" t="n"/>
+      <c r="G121" s="5" t="n"/>
     </row>
     <row r="122" ht="18" customHeight="1">
       <c r="A122" s="20" t="inlineStr">
         <is>
-          <t>Main Bar:</t>
+          <t>Waters:</t>
         </is>
       </c>
       <c r="B122" s="5" t="n"/>
-      <c r="C122" s="20" t="inlineStr">
-        <is>
-          <t>On tonight:</t>
-        </is>
-      </c>
-      <c r="D122" s="5" t="n"/>
       <c r="E122" s="20" t="inlineStr">
         <is>
-          <t>Running it:</t>
+          <t>200:</t>
         </is>
       </c>
       <c r="F122" s="5" t="n"/>
@@ -1937,46 +1958,76 @@
     <row r="123" ht="18" customHeight="1">
       <c r="A123" s="20" t="inlineStr">
         <is>
-          <t>Patio Bar:</t>
+          <t>Bathrooms:</t>
         </is>
       </c>
       <c r="B123" s="5" t="n"/>
-    </row>
-    <row r="124" ht="18" customHeight="1">
-      <c r="A124" s="20" t="inlineStr">
-        <is>
-          <t>Main Floor:</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="n"/>
-    </row>
-    <row r="125" ht="18" customHeight="1">
-      <c r="A125" s="20" t="inlineStr">
-        <is>
-          <t>Café:</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="n"/>
+      <c r="E123" s="20" t="inlineStr">
+        <is>
+          <t>Patio:</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="n"/>
+      <c r="G123" s="5" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
+          <t>BARBACKS</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>SHOT GIRL</t>
+        </is>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t>TASTE PLATE</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="20" t="inlineStr">
         <is>
-          <t>Front Patio:</t>
+          <t>Main Bar:</t>
         </is>
       </c>
       <c r="B126" s="5" t="n"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="inlineStr">
-        <is>
-          <t>SOCIAL MEDIA</t>
-        </is>
-      </c>
+      <c r="C126" s="20" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="n"/>
+      <c r="E126" s="20" t="inlineStr">
+        <is>
+          <t>Running it:</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="n"/>
+      <c r="G126" s="5" t="n"/>
+    </row>
+    <row r="127" ht="18" customHeight="1">
+      <c r="A127" s="20" t="inlineStr">
+        <is>
+          <t>Patio Bar:</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="n"/>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="A128" s="20" t="inlineStr">
+        <is>
+          <t>Main Floor:</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="n"/>
     </row>
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="20" t="inlineStr">
         <is>
-          <t>On tonight:</t>
+          <t>Café:</t>
         </is>
       </c>
       <c r="B129" s="5" t="n"/>
@@ -1984,473 +2035,496 @@
     <row r="130" ht="18" customHeight="1">
       <c r="A130" s="20" t="inlineStr">
         <is>
+          <t>Front Patio:</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL MEDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="A133" s="20" t="inlineStr">
+        <is>
+          <t>On tonight:</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="n"/>
+    </row>
+    <row r="134" ht="18" customHeight="1">
+      <c r="A134" s="20" t="inlineStr">
+        <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B130" s="5" t="n"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="4" t="inlineStr">
+      <c r="B134" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
         <is>
           <t>PARTIES / EVENTS:</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="16" t="n"/>
-      <c r="B134" s="17" t="n"/>
-      <c r="C134" s="17" t="n"/>
-      <c r="D134" s="17" t="n"/>
-      <c r="E134" s="17" t="n"/>
-      <c r="F134" s="17" t="n"/>
-      <c r="G134" s="17" t="n"/>
-    </row>
-    <row r="135" ht="18" customHeight="1">
-      <c r="A135" s="17" t="n"/>
-      <c r="B135" s="17" t="n"/>
-      <c r="C135" s="17" t="n"/>
-      <c r="D135" s="17" t="n"/>
-      <c r="E135" s="17" t="n"/>
-      <c r="F135" s="17" t="n"/>
-      <c r="G135" s="17" t="n"/>
-    </row>
-    <row r="137" ht="18" customHeight="1">
-      <c r="A137" s="6" t="inlineStr">
+    <row r="138" ht="18" customHeight="1">
+      <c r="A138" s="16" t="n"/>
+      <c r="B138" s="17" t="n"/>
+      <c r="C138" s="17" t="n"/>
+      <c r="D138" s="17" t="n"/>
+      <c r="E138" s="17" t="n"/>
+      <c r="F138" s="17" t="n"/>
+      <c r="G138" s="17" t="n"/>
+    </row>
+    <row r="139" ht="18" customHeight="1">
+      <c r="A139" s="17" t="n"/>
+      <c r="B139" s="17" t="n"/>
+      <c r="C139" s="17" t="n"/>
+      <c r="D139" s="17" t="n"/>
+      <c r="E139" s="17" t="n"/>
+      <c r="F139" s="17" t="n"/>
+      <c r="G139" s="17" t="n"/>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="6" t="inlineStr">
         <is>
           <t>GAME DAY OPEN — 90 MINUTES BEFORE DOORS</t>
         </is>
       </c>
-      <c r="B137" s="7" t="n"/>
-      <c r="C137" s="7" t="n"/>
-      <c r="D137" s="7" t="n"/>
-      <c r="E137" s="7" t="n"/>
-      <c r="F137" s="7" t="n"/>
-      <c r="G137" s="7" t="n"/>
-    </row>
-    <row r="138" ht="17" customHeight="1">
-      <c r="A138" s="21" t="inlineStr">
+      <c r="B141" s="7" t="n"/>
+      <c r="C141" s="7" t="n"/>
+      <c r="D141" s="7" t="n"/>
+      <c r="E141" s="7" t="n"/>
+      <c r="F141" s="7" t="n"/>
+      <c r="G141" s="7" t="n"/>
+    </row>
+    <row r="142" ht="17" customHeight="1">
+      <c r="A142" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B138" s="9" t="inlineStr">
+      <c r="B142" s="9" t="inlineStr">
         <is>
           <t>Know the game — kickoff, attendance, national TV, weather. Times on the board.</t>
         </is>
       </c>
     </row>
-    <row r="139" ht="17" customHeight="1">
-      <c r="A139" s="21" t="inlineStr">
+    <row r="143" ht="17" customHeight="1">
+      <c r="A143" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B139" s="9" t="inlineStr">
+      <c r="B143" s="9" t="inlineStr">
         <is>
           <t>Every staff member can name all three promos — ask two people at random before pre-shift ends.</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="17" customHeight="1">
-      <c r="A140" s="21" t="inlineStr">
+    <row r="144" ht="17" customHeight="1">
+      <c r="A144" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B140" s="9" t="inlineStr">
+      <c r="B144" s="9" t="inlineStr">
         <is>
           <t>Anthem time on the board — every staff member knows to line up behind the bar.</t>
         </is>
       </c>
     </row>
-    <row r="141" ht="17" customHeight="1">
-      <c r="A141" s="21" t="inlineStr">
+    <row r="145" ht="17" customHeight="1">
+      <c r="A145" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B141" s="9" t="inlineStr">
+      <c r="B145" s="9" t="inlineStr">
         <is>
           <t>Social media assigned, phone charged, and they know the shot list.</t>
         </is>
       </c>
     </row>
-    <row r="142" ht="17" customHeight="1">
-      <c r="A142" s="21" t="inlineStr">
+    <row r="146" ht="17" customHeight="1">
+      <c r="A146" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B142" s="9" t="inlineStr">
+      <c r="B146" s="9" t="inlineStr">
         <is>
           <t>Three windows built on paper — cut times, breaks, post-game all-hands decided now.</t>
         </is>
       </c>
     </row>
-    <row r="143" ht="17" customHeight="1">
-      <c r="A143" s="21" t="inlineStr">
+    <row r="147" ht="17" customHeight="1">
+      <c r="A147" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B143" s="9" t="inlineStr">
+      <c r="B147" s="9" t="inlineStr">
         <is>
           <t>Staffing confirmed against 7shifts. One no-show on game day is a two-hour wait.</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="17" customHeight="1">
-      <c r="A144" s="21" t="inlineStr">
+    <row r="148" ht="17" customHeight="1">
+      <c r="A148" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B144" s="9" t="inlineStr">
+      <c r="B148" s="9" t="inlineStr">
         <is>
           <t>Every station walked, front and back. The 3 Rules on all of them.</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="17" customHeight="1">
-      <c r="A145" s="21" t="inlineStr">
+    <row r="149" ht="17" customHeight="1">
+      <c r="A149" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B145" s="9" t="inlineStr">
+      <c r="B149" s="9" t="inlineStr">
         <is>
           <t>Bar par DOUBLED — ice, kegs, backups, garnish, glassware, batch.</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="17" customHeight="1">
-      <c r="A146" s="21" t="inlineStr">
+    <row r="150" ht="17" customHeight="1">
+      <c r="A150" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B146" s="9" t="inlineStr">
+      <c r="B150" s="9" t="inlineStr">
         <is>
           <t>86 board walked with the kitchen, current and visible.</t>
         </is>
       </c>
     </row>
-    <row r="147" ht="17" customHeight="1">
-      <c r="A147" s="21" t="inlineStr">
+    <row r="151" ht="17" customHeight="1">
+      <c r="A151" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B147" s="9" t="inlineStr">
+      <c r="B151" s="9" t="inlineStr">
         <is>
           <t>TVs, sound and the game feed tested before a single guest sits down.</t>
         </is>
       </c>
     </row>
-    <row r="148" ht="17" customHeight="1">
-      <c r="A148" s="21" t="inlineStr">
+    <row r="152" ht="17" customHeight="1">
+      <c r="A152" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B148" s="9" t="inlineStr">
+      <c r="B152" s="9" t="inlineStr">
         <is>
           <t>ID check covered — door and bar know who is carding, and the light works.</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="17" customHeight="1">
-      <c r="A149" s="21" t="inlineStr">
+    <row r="153" ht="17" customHeight="1">
+      <c r="A153" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B149" s="9" t="inlineStr">
+      <c r="B153" s="9" t="inlineStr">
         <is>
           <t>Restrooms stocked and clean before doors.</t>
         </is>
       </c>
     </row>
-    <row r="150" ht="17" customHeight="1">
-      <c r="A150" s="21" t="inlineStr">
+    <row r="154" ht="17" customHeight="1">
+      <c r="A154" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B150" s="9" t="inlineStr">
+      <c r="B154" s="9" t="inlineStr">
         <is>
           <t>POS, printers and card processing tested with a live ticket.</t>
         </is>
       </c>
     </row>
-    <row r="151" ht="17" customHeight="1">
-      <c r="A151" s="21" t="inlineStr">
+    <row r="155" ht="17" customHeight="1">
+      <c r="A155" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B151" s="9" t="inlineStr">
+      <c r="B155" s="9" t="inlineStr">
         <is>
           <t>Cash on hand for a bar that will run cash all night.</t>
         </is>
       </c>
     </row>
-    <row r="152" ht="17" customHeight="1">
-      <c r="A152" s="21" t="inlineStr">
+    <row r="156" ht="17" customHeight="1">
+      <c r="A156" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B152" s="9" t="inlineStr">
+      <c r="B156" s="9" t="inlineStr">
         <is>
           <t>Door, patio and line plan — where the wait forms and who holds it.</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="20" customHeight="1">
-      <c r="A154" s="22" t="inlineStr">
+    <row r="158" ht="20" customHeight="1">
+      <c r="A158" s="25" t="inlineStr">
         <is>
           <t>IS STAFF IN UNIFORM?   YES / NO</t>
         </is>
       </c>
-      <c r="B154" s="13" t="n"/>
-      <c r="C154" s="13" t="n"/>
-      <c r="D154" s="22" t="inlineStr">
+      <c r="B158" s="13" t="n"/>
+      <c r="C158" s="13" t="n"/>
+      <c r="D158" s="25" t="inlineStr">
         <is>
           <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
         </is>
       </c>
-      <c r="E154" s="13" t="n"/>
-      <c r="F154" s="13" t="n"/>
-      <c r="G154" s="13" t="n"/>
-    </row>
-    <row r="155" ht="20" customHeight="1">
-      <c r="A155" s="22" t="inlineStr">
+      <c r="E158" s="13" t="n"/>
+      <c r="F158" s="13" t="n"/>
+      <c r="G158" s="13" t="n"/>
+    </row>
+    <row r="159" ht="20" customHeight="1">
+      <c r="A159" s="25" t="inlineStr">
         <is>
           <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
         </is>
       </c>
-      <c r="B155" s="13" t="n"/>
-      <c r="C155" s="13" t="n"/>
-      <c r="D155" s="22" t="inlineStr">
+      <c r="B159" s="13" t="n"/>
+      <c r="C159" s="13" t="n"/>
+      <c r="D159" s="25" t="inlineStr">
         <is>
           <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
         </is>
       </c>
-      <c r="E155" s="13" t="n"/>
-      <c r="F155" s="13" t="n"/>
-      <c r="G155" s="13" t="n"/>
-    </row>
-    <row r="156" ht="20" customHeight="1">
-      <c r="A156" s="22" t="inlineStr">
+      <c r="E159" s="13" t="n"/>
+      <c r="F159" s="13" t="n"/>
+      <c r="G159" s="13" t="n"/>
+    </row>
+    <row r="160" ht="20" customHeight="1">
+      <c r="A160" s="25" t="inlineStr">
         <is>
           <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
         </is>
       </c>
-      <c r="B156" s="13" t="n"/>
-      <c r="C156" s="13" t="n"/>
-      <c r="D156" s="13" t="n"/>
-      <c r="E156" s="13" t="n"/>
-      <c r="F156" s="13" t="n"/>
-      <c r="G156" s="13" t="n"/>
-    </row>
-    <row r="158" ht="18" customHeight="1">
-      <c r="A158" s="6" t="inlineStr">
+      <c r="B160" s="13" t="n"/>
+      <c r="C160" s="13" t="n"/>
+      <c r="D160" s="13" t="n"/>
+      <c r="E160" s="13" t="n"/>
+      <c r="F160" s="13" t="n"/>
+      <c r="G160" s="13" t="n"/>
+    </row>
+    <row r="162" ht="18" customHeight="1">
+      <c r="A162" s="6" t="inlineStr">
         <is>
           <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
         </is>
       </c>
-      <c r="B158" s="7" t="n"/>
-      <c r="C158" s="7" t="n"/>
-      <c r="D158" s="7" t="n"/>
-      <c r="E158" s="7" t="n"/>
-      <c r="F158" s="7" t="n"/>
-      <c r="G158" s="7" t="n"/>
-    </row>
-    <row r="159" ht="32" customHeight="1">
-      <c r="A159" s="8" t="inlineStr">
-        <is>
-          <t>BAR</t>
-        </is>
-      </c>
-      <c r="B159" s="9" t="inlineStr">
-        <is>
-          <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="32" customHeight="1">
-      <c r="A160" s="8" t="inlineStr">
-        <is>
-          <t>SERVERS</t>
-        </is>
-      </c>
-      <c r="B160" s="9" t="inlineStr">
-        <is>
-          <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161" ht="32" customHeight="1">
-      <c r="A161" s="8" t="inlineStr">
-        <is>
-          <t>HOST</t>
-        </is>
-      </c>
-      <c r="B161" s="9" t="inlineStr">
-        <is>
-          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. First in command runs the book; second in command steps in the moment first gets pulled. Card at the door when the room is young. Keep the line off the sidewalk and feed the wait to the bar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162" ht="32" customHeight="1">
-      <c r="A162" s="8" t="inlineStr">
-        <is>
-          <t>KITCHEN</t>
-        </is>
-      </c>
-      <c r="B162" s="9" t="inlineStr">
-        <is>
-          <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
-        </is>
-      </c>
+      <c r="B162" s="7" t="n"/>
+      <c r="C162" s="7" t="n"/>
+      <c r="D162" s="7" t="n"/>
+      <c r="E162" s="7" t="n"/>
+      <c r="F162" s="7" t="n"/>
+      <c r="G162" s="7" t="n"/>
     </row>
     <row r="163" ht="32" customHeight="1">
       <c r="A163" s="8" t="inlineStr">
         <is>
-          <t>SOCIAL</t>
+          <t>BAR</t>
         </is>
       </c>
       <c r="B163" s="9" t="inlineStr">
         <is>
-          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
+          <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
         </is>
       </c>
     </row>
     <row r="164" ht="32" customHeight="1">
       <c r="A164" s="8" t="inlineStr">
         <is>
+          <t>SERVERS</t>
+        </is>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="32" customHeight="1">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t>HOST</t>
+        </is>
+      </c>
+      <c r="B165" s="9" t="inlineStr">
+        <is>
+          <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. First in command runs the book; second in command steps in the moment first gets pulled. Card at the door when the room is young. Keep the line off the sidewalk and feed the wait to the bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="32" customHeight="1">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t>KITCHEN</t>
+        </is>
+      </c>
+      <c r="B166" s="9" t="inlineStr">
+        <is>
+          <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="32" customHeight="1">
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>SOCIAL</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="32" customHeight="1">
+      <c r="A168" s="8" t="inlineStr">
+        <is>
           <t>SUPPORT</t>
         </is>
       </c>
-      <c r="B164" s="9" t="inlineStr">
+      <c r="B168" s="9" t="inlineStr">
         <is>
           <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
         </is>
       </c>
     </row>
-    <row r="166" ht="18" customHeight="1">
-      <c r="A166" s="6" t="inlineStr">
+    <row r="170" ht="18" customHeight="1">
+      <c r="A170" s="6" t="inlineStr">
         <is>
           <t>POST-GAME &amp; CLOSE</t>
         </is>
       </c>
-      <c r="B166" s="7" t="n"/>
-      <c r="C166" s="7" t="n"/>
-      <c r="D166" s="7" t="n"/>
-      <c r="E166" s="7" t="n"/>
-      <c r="F166" s="7" t="n"/>
-      <c r="G166" s="7" t="n"/>
-    </row>
-    <row r="167" ht="17" customHeight="1">
-      <c r="A167" s="21" t="inlineStr">
+      <c r="B170" s="7" t="n"/>
+      <c r="C170" s="7" t="n"/>
+      <c r="D170" s="7" t="n"/>
+      <c r="E170" s="7" t="n"/>
+      <c r="F170" s="7" t="n"/>
+      <c r="G170" s="7" t="n"/>
+    </row>
+    <row r="171" ht="17" customHeight="1">
+      <c r="A171" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B167" s="9" t="inlineStr">
+      <c r="B171" s="9" t="inlineStr">
         <is>
           <t>All hands on the floor BEFORE the final whistle — not after.</t>
         </is>
       </c>
     </row>
-    <row r="168" ht="17" customHeight="1">
-      <c r="A168" s="21" t="inlineStr">
+    <row r="172" ht="17" customHeight="1">
+      <c r="A172" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B168" s="9" t="inlineStr">
+      <c r="B172" s="9" t="inlineStr">
         <is>
           <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
         </is>
       </c>
     </row>
-    <row r="169" ht="17" customHeight="1">
-      <c r="A169" s="21" t="inlineStr">
+    <row r="173" ht="17" customHeight="1">
+      <c r="A173" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B169" s="9" t="inlineStr">
+      <c r="B173" s="9" t="inlineStr">
         <is>
           <t>Every void, comp and discount reconciled to a manager name.</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="17" customHeight="1">
-      <c r="A170" s="21" t="inlineStr">
+    <row r="174" ht="17" customHeight="1">
+      <c r="A174" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B170" s="9" t="inlineStr">
+      <c r="B174" s="9" t="inlineStr">
         <is>
           <t>Every refusal or cut-off logged with what happened and who made the call.</t>
         </is>
       </c>
     </row>
-    <row r="171" ht="17" customHeight="1">
-      <c r="A171" s="21" t="inlineStr">
+    <row r="175" ht="17" customHeight="1">
+      <c r="A175" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B171" s="9" t="inlineStr">
+      <c r="B175" s="9" t="inlineStr">
         <is>
           <t>Every station back to original position, original condition.</t>
         </is>
       </c>
     </row>
-    <row r="172" ht="17" customHeight="1">
-      <c r="A172" s="21" t="inlineStr">
+    <row r="176" ht="17" customHeight="1">
+      <c r="A176" s="24" t="inlineStr">
         <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="B172" s="9" t="inlineStr">
+      <c r="B176" s="9" t="inlineStr">
         <is>
           <t>Shift notes written: what we ran out of, where the wait broke down, what changes next game.</t>
         </is>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="4" t="inlineStr">
+    <row r="178">
+      <c r="A178" s="4" t="inlineStr">
         <is>
           <t>MARKETING:</t>
         </is>
       </c>
     </row>
-    <row r="175" ht="18" customHeight="1">
-      <c r="A175" s="16" t="n"/>
-      <c r="B175" s="17" t="n"/>
-      <c r="C175" s="17" t="n"/>
-      <c r="D175" s="17" t="n"/>
-      <c r="E175" s="17" t="n"/>
-      <c r="F175" s="17" t="n"/>
-      <c r="G175" s="17" t="n"/>
-    </row>
-    <row r="176" ht="18" customHeight="1">
-      <c r="A176" s="17" t="n"/>
-      <c r="B176" s="17" t="n"/>
-      <c r="C176" s="17" t="n"/>
-      <c r="D176" s="17" t="n"/>
-      <c r="E176" s="17" t="n"/>
-      <c r="F176" s="17" t="n"/>
-      <c r="G176" s="17" t="n"/>
-    </row>
-    <row r="178" ht="28" customHeight="1">
-      <c r="A178" s="23" t="inlineStr">
+    <row r="179" ht="18" customHeight="1">
+      <c r="A179" s="16" t="n"/>
+      <c r="B179" s="17" t="n"/>
+      <c r="C179" s="17" t="n"/>
+      <c r="D179" s="17" t="n"/>
+      <c r="E179" s="17" t="n"/>
+      <c r="F179" s="17" t="n"/>
+      <c r="G179" s="17" t="n"/>
+    </row>
+    <row r="180" ht="18" customHeight="1">
+      <c r="A180" s="17" t="n"/>
+      <c r="B180" s="17" t="n"/>
+      <c r="C180" s="17" t="n"/>
+      <c r="D180" s="17" t="n"/>
+      <c r="E180" s="17" t="n"/>
+      <c r="F180" s="17" t="n"/>
+      <c r="G180" s="17" t="n"/>
+    </row>
+    <row r="182" ht="28" customHeight="1">
+      <c r="A182" s="26" t="inlineStr">
         <is>
           <t>100% of our standards, 100% of the time, at 100% volume. A full house is not an excuse to run at 80% — it is the reason we hold the line.</t>
         </is>
@@ -2460,58 +2534,58 @@
   <mergeCells count="73">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A141:G141"/>
+    <mergeCell ref="A97:G97"/>
     <mergeCell ref="B145:G145"/>
     <mergeCell ref="B151:G151"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A22:G22"/>
-    <mergeCell ref="B170:G170"/>
     <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A96:G96"/>
     <mergeCell ref="B148:G148"/>
-    <mergeCell ref="A156:G156"/>
+    <mergeCell ref="A158:C158"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A154:C154"/>
+    <mergeCell ref="B166:G166"/>
+    <mergeCell ref="B175:G175"/>
     <mergeCell ref="B171:G171"/>
     <mergeCell ref="D51:G51"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="B147:G147"/>
-    <mergeCell ref="B162:G162"/>
+    <mergeCell ref="A170:G170"/>
     <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A93:G93"/>
+    <mergeCell ref="A117:G117"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="B172:G172"/>
+    <mergeCell ref="B174:G174"/>
     <mergeCell ref="B168:G168"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="B146:G146"/>
-    <mergeCell ref="A92:G92"/>
+    <mergeCell ref="A159:C159"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="B143:G143"/>
-    <mergeCell ref="A166:G166"/>
+    <mergeCell ref="A179:G180"/>
     <mergeCell ref="C9:G9"/>
-    <mergeCell ref="B139:G139"/>
-    <mergeCell ref="A178:G178"/>
+    <mergeCell ref="A182:G182"/>
+    <mergeCell ref="D159:G159"/>
     <mergeCell ref="B142:G142"/>
-    <mergeCell ref="D155:G155"/>
     <mergeCell ref="B164:G164"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A134:G135"/>
-    <mergeCell ref="A155:C155"/>
-    <mergeCell ref="A158:G158"/>
-    <mergeCell ref="B160:G160"/>
-    <mergeCell ref="B169:G169"/>
-    <mergeCell ref="A175:G176"/>
+    <mergeCell ref="D158:G158"/>
+    <mergeCell ref="A162:G162"/>
+    <mergeCell ref="B154:G154"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="A47:G48"/>
     <mergeCell ref="B163:G163"/>
     <mergeCell ref="B144:G144"/>
+    <mergeCell ref="B173:G173"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="B138:G138"/>
-    <mergeCell ref="A137:G137"/>
+    <mergeCell ref="B153:G153"/>
+    <mergeCell ref="A160:G160"/>
+    <mergeCell ref="B165:G165"/>
     <mergeCell ref="A35:G36"/>
-    <mergeCell ref="D154:G154"/>
-    <mergeCell ref="A74:G74"/>
-    <mergeCell ref="B141:G141"/>
+    <mergeCell ref="B156:G156"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A56:G56"/>
@@ -2521,15 +2595,15 @@
     <mergeCell ref="B150:G150"/>
     <mergeCell ref="A50:G50"/>
     <mergeCell ref="A39:G40"/>
-    <mergeCell ref="B140:G140"/>
+    <mergeCell ref="B155:G155"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="B149:G149"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B159:G159"/>
     <mergeCell ref="B167:G167"/>
-    <mergeCell ref="A113:G113"/>
-    <mergeCell ref="B161:G161"/>
+    <mergeCell ref="A76:G76"/>
+    <mergeCell ref="B176:G176"/>
     <mergeCell ref="B152:G152"/>
+    <mergeCell ref="A138:G139"/>
     <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add a barista station to the assignments grid
Barista sits between Bar and Barbacks with four lines — POS 1, POS 2,
Cocktail 1 and Cocktail 2 — in both the AM and PM crews. The two POS lines
are numbered so a manager can tell which is which when filling the sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -1763,36 +1763,36 @@
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
+          <t>BARISTA</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
           <t>BARBACKS</t>
         </is>
       </c>
-      <c r="C105" s="8" t="inlineStr">
+      <c r="E105" s="8" t="inlineStr">
         <is>
           <t>SHOT GIRL</t>
-        </is>
-      </c>
-      <c r="E105" s="8" t="inlineStr">
-        <is>
-          <t>TASTE PLATE</t>
         </is>
       </c>
     </row>
     <row r="106" ht="18" customHeight="1">
       <c r="A106" s="20" t="inlineStr">
         <is>
-          <t>Main Bar:</t>
+          <t>POS 1:</t>
         </is>
       </c>
       <c r="B106" s="5" t="n"/>
       <c r="C106" s="20" t="inlineStr">
         <is>
-          <t>On tonight:</t>
+          <t>Main Bar:</t>
         </is>
       </c>
       <c r="D106" s="5" t="n"/>
       <c r="E106" s="20" t="inlineStr">
         <is>
-          <t>Running it:</t>
+          <t>On tonight:</t>
         </is>
       </c>
       <c r="F106" s="5" t="n"/>
@@ -1801,38 +1801,61 @@
     <row r="107" ht="18" customHeight="1">
       <c r="A107" s="20" t="inlineStr">
         <is>
+          <t>POS 2:</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="n"/>
+      <c r="C107" s="20" t="inlineStr">
+        <is>
           <t>Patio Bar:</t>
         </is>
       </c>
-      <c r="B107" s="5" t="n"/>
+      <c r="D107" s="5" t="n"/>
     </row>
     <row r="108" ht="18" customHeight="1">
       <c r="A108" s="20" t="inlineStr">
         <is>
+          <t>Cocktail 1:</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="n"/>
+      <c r="C108" s="20" t="inlineStr">
+        <is>
           <t>Main Floor:</t>
         </is>
       </c>
-      <c r="B108" s="5" t="n"/>
+      <c r="D108" s="5" t="n"/>
     </row>
     <row r="109" ht="18" customHeight="1">
       <c r="A109" s="20" t="inlineStr">
         <is>
+          <t>Cocktail 2:</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="n"/>
+      <c r="C109" s="20" t="inlineStr">
+        <is>
           <t>Café:</t>
         </is>
       </c>
-      <c r="B109" s="5" t="n"/>
+      <c r="D109" s="5" t="n"/>
     </row>
     <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="20" t="inlineStr">
+      <c r="C110" s="20" t="inlineStr">
         <is>
           <t>Front Patio:</t>
         </is>
       </c>
-      <c r="B110" s="5" t="n"/>
+      <c r="D110" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="8" t="inlineStr">
         <is>
+          <t>TASTE PLATE</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
           <t>SOCIAL MEDIA</t>
         </is>
       </c>
@@ -1840,18 +1863,24 @@
     <row r="113" ht="18" customHeight="1">
       <c r="A113" s="20" t="inlineStr">
         <is>
+          <t>Running it:</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="n"/>
+      <c r="C113" s="20" t="inlineStr">
+        <is>
           <t>On tonight:</t>
         </is>
       </c>
-      <c r="B113" s="5" t="n"/>
+      <c r="D113" s="5" t="n"/>
     </row>
     <row r="114" ht="18" customHeight="1">
-      <c r="A114" s="20" t="inlineStr">
+      <c r="C114" s="20" t="inlineStr">
         <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B114" s="5" t="n"/>
+      <c r="D114" s="5" t="n"/>
     </row>
     <row r="117" ht="17" customHeight="1">
       <c r="A117" s="8" t="inlineStr">
@@ -1973,36 +2002,36 @@
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
+          <t>BARISTA</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
           <t>BARBACKS</t>
         </is>
       </c>
-      <c r="C125" s="8" t="inlineStr">
+      <c r="E125" s="8" t="inlineStr">
         <is>
           <t>SHOT GIRL</t>
-        </is>
-      </c>
-      <c r="E125" s="8" t="inlineStr">
-        <is>
-          <t>TASTE PLATE</t>
         </is>
       </c>
     </row>
     <row r="126" ht="18" customHeight="1">
       <c r="A126" s="20" t="inlineStr">
         <is>
-          <t>Main Bar:</t>
+          <t>POS 1:</t>
         </is>
       </c>
       <c r="B126" s="5" t="n"/>
       <c r="C126" s="20" t="inlineStr">
         <is>
-          <t>On tonight:</t>
+          <t>Main Bar:</t>
         </is>
       </c>
       <c r="D126" s="5" t="n"/>
       <c r="E126" s="20" t="inlineStr">
         <is>
-          <t>Running it:</t>
+          <t>On tonight:</t>
         </is>
       </c>
       <c r="F126" s="5" t="n"/>
@@ -2011,38 +2040,61 @@
     <row r="127" ht="18" customHeight="1">
       <c r="A127" s="20" t="inlineStr">
         <is>
+          <t>POS 2:</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="n"/>
+      <c r="C127" s="20" t="inlineStr">
+        <is>
           <t>Patio Bar:</t>
         </is>
       </c>
-      <c r="B127" s="5" t="n"/>
+      <c r="D127" s="5" t="n"/>
     </row>
     <row r="128" ht="18" customHeight="1">
       <c r="A128" s="20" t="inlineStr">
         <is>
+          <t>Cocktail 1:</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="n"/>
+      <c r="C128" s="20" t="inlineStr">
+        <is>
           <t>Main Floor:</t>
         </is>
       </c>
-      <c r="B128" s="5" t="n"/>
+      <c r="D128" s="5" t="n"/>
     </row>
     <row r="129" ht="18" customHeight="1">
       <c r="A129" s="20" t="inlineStr">
         <is>
+          <t>Cocktail 2:</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="n"/>
+      <c r="C129" s="20" t="inlineStr">
+        <is>
           <t>Café:</t>
         </is>
       </c>
-      <c r="B129" s="5" t="n"/>
+      <c r="D129" s="5" t="n"/>
     </row>
     <row r="130" ht="18" customHeight="1">
-      <c r="A130" s="20" t="inlineStr">
+      <c r="C130" s="20" t="inlineStr">
         <is>
           <t>Front Patio:</t>
         </is>
       </c>
-      <c r="B130" s="5" t="n"/>
+      <c r="D130" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
+          <t>TASTE PLATE</t>
+        </is>
+      </c>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
           <t>SOCIAL MEDIA</t>
         </is>
       </c>
@@ -2050,18 +2102,24 @@
     <row r="133" ht="18" customHeight="1">
       <c r="A133" s="20" t="inlineStr">
         <is>
+          <t>Running it:</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="n"/>
+      <c r="C133" s="20" t="inlineStr">
+        <is>
           <t>On tonight:</t>
         </is>
       </c>
-      <c r="B133" s="5" t="n"/>
+      <c r="D133" s="5" t="n"/>
     </row>
     <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="20" t="inlineStr">
+      <c r="C134" s="20" t="inlineStr">
         <is>
           <t>Backup / 2nd half:</t>
         </is>
       </c>
-      <c r="B134" s="5" t="n"/>
+      <c r="D134" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Replace the uniform yes/no with a uniform check
"Is staff in uniform?" was one box for eight separate standards. It is now its
own tickable list: OSU body suit and/or polo, eye black, glitter, ribbon,
hair, makeup done, hair done, and gentlemen have a belt on.

The remaining yes/no row keeps wine key and lighter, ID'ing, TVs and game
feed, and bar par — the workbook and the page now carry the same four.

No field keys were renamed; existing entries are untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0141fQgW8SdSU55Py26WqSNq
</commit_message>
<xml_diff>
--- a/docs/GameDay_PreShift_Template.xlsx
+++ b/docs/GameDay_PreShift_Template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Game Day Pre-Shift" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$182</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Game Day Pre-Shift'!$A$1:$G$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G182"/>
+  <dimension ref="A1:G192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.5" customWidth="1" min="1" max="1"/>
@@ -2339,330 +2339,448 @@
         </is>
       </c>
     </row>
-    <row r="158" ht="20" customHeight="1">
-      <c r="A158" s="25" t="inlineStr">
-        <is>
-          <t>IS STAFF IN UNIFORM?   YES / NO</t>
-        </is>
-      </c>
-      <c r="B158" s="13" t="n"/>
-      <c r="C158" s="13" t="n"/>
-      <c r="D158" s="25" t="inlineStr">
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="6" t="inlineStr">
+        <is>
+          <t>UNIFORM CHECK</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="n"/>
+      <c r="C158" s="7" t="n"/>
+      <c r="D158" s="7" t="n"/>
+      <c r="E158" s="7" t="n"/>
+      <c r="F158" s="7" t="n"/>
+      <c r="G158" s="7" t="n"/>
+    </row>
+    <row r="159" ht="17" customHeight="1">
+      <c r="A159" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>OSU body suit and / or polo</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="17" customHeight="1">
+      <c r="A160" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>Eye black</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="17" customHeight="1">
+      <c r="A161" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B161" s="9" t="inlineStr">
+        <is>
+          <t>Glitter</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="17" customHeight="1">
+      <c r="A162" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>Ribbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="17" customHeight="1">
+      <c r="A163" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>Hair</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="17" customHeight="1">
+      <c r="A164" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>Makeup done</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="17" customHeight="1">
+      <c r="A165" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B165" s="9" t="inlineStr">
+        <is>
+          <t>Hair done</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="17" customHeight="1">
+      <c r="A166" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B166" s="9" t="inlineStr">
+        <is>
+          <t>Gentlemen have a belt on</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="25" t="inlineStr">
         <is>
           <t>SERVERS HAVE WINE KEY &amp; LIGHTER?   YES / NO</t>
         </is>
       </c>
-      <c r="E158" s="13" t="n"/>
-      <c r="F158" s="13" t="n"/>
-      <c r="G158" s="13" t="n"/>
-    </row>
-    <row r="159" ht="20" customHeight="1">
-      <c r="A159" s="25" t="inlineStr">
+      <c r="B168" s="13" t="n"/>
+      <c r="C168" s="13" t="n"/>
+      <c r="D168" s="25" t="inlineStr">
         <is>
           <t>ID'ING EVERYONE UNDER 40?   YES / NO</t>
         </is>
       </c>
-      <c r="B159" s="13" t="n"/>
-      <c r="C159" s="13" t="n"/>
-      <c r="D159" s="25" t="inlineStr">
+      <c r="E168" s="13" t="n"/>
+      <c r="F168" s="13" t="n"/>
+      <c r="G168" s="13" t="n"/>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="A169" s="25" t="inlineStr">
         <is>
           <t>TVs &amp; GAME FEED TESTED?   YES / NO</t>
         </is>
       </c>
-      <c r="E159" s="13" t="n"/>
-      <c r="F159" s="13" t="n"/>
-      <c r="G159" s="13" t="n"/>
-    </row>
-    <row r="160" ht="20" customHeight="1">
-      <c r="A160" s="25" t="inlineStr">
+      <c r="B169" s="13" t="n"/>
+      <c r="C169" s="13" t="n"/>
+      <c r="D169" s="25" t="inlineStr">
+        <is>
+          <t>BAR PAR DOUBLED FOR POST-GAME?   YES / NO</t>
+        </is>
+      </c>
+      <c r="E169" s="13" t="n"/>
+      <c r="F169" s="13" t="n"/>
+      <c r="G169" s="13" t="n"/>
+    </row>
+    <row r="170" ht="20" customHeight="1">
+      <c r="A170" s="25" t="inlineStr">
         <is>
           <t>**REMIND STAFF TO TEXT FRIENDS TO COME VISIT**</t>
         </is>
       </c>
-      <c r="B160" s="13" t="n"/>
-      <c r="C160" s="13" t="n"/>
-      <c r="D160" s="13" t="n"/>
-      <c r="E160" s="13" t="n"/>
-      <c r="F160" s="13" t="n"/>
-      <c r="G160" s="13" t="n"/>
-    </row>
-    <row r="162" ht="18" customHeight="1">
-      <c r="A162" s="6" t="inlineStr">
+      <c r="B170" s="13" t="n"/>
+      <c r="C170" s="13" t="n"/>
+      <c r="D170" s="13" t="n"/>
+      <c r="E170" s="13" t="n"/>
+      <c r="F170" s="13" t="n"/>
+      <c r="G170" s="13" t="n"/>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="6" t="inlineStr">
         <is>
           <t>BY POSITION — READ THE BLOCK THAT BELONGS TO EACH GROUP</t>
         </is>
       </c>
-      <c r="B162" s="7" t="n"/>
-      <c r="C162" s="7" t="n"/>
-      <c r="D162" s="7" t="n"/>
-      <c r="E162" s="7" t="n"/>
-      <c r="F162" s="7" t="n"/>
-      <c r="G162" s="7" t="n"/>
-    </row>
-    <row r="163" ht="32" customHeight="1">
-      <c r="A163" s="8" t="inlineStr">
+      <c r="B172" s="7" t="n"/>
+      <c r="C172" s="7" t="n"/>
+      <c r="D172" s="7" t="n"/>
+      <c r="E172" s="7" t="n"/>
+      <c r="F172" s="7" t="n"/>
+      <c r="G172" s="7" t="n"/>
+    </row>
+    <row r="173" ht="32" customHeight="1">
+      <c r="A173" s="8" t="inlineStr">
         <is>
           <t>BAR</t>
         </is>
       </c>
-      <c r="B163" s="9" t="inlineStr">
+      <c r="B173" s="9" t="inlineStr">
         <is>
           <t>ID before you pour — every time, no exceptions. Every drink rings before it pours. No promo bottles, no comps. Cut people early and tell a manager immediately. Stock backups during the game window, not after it.</t>
         </is>
       </c>
     </row>
-    <row r="164" ht="32" customHeight="1">
-      <c r="A164" s="8" t="inlineStr">
+    <row r="174" ht="32" customHeight="1">
+      <c r="A174" s="8" t="inlineStr">
         <is>
           <t>SERVERS</t>
         </is>
       </c>
-      <c r="B164" s="9" t="inlineStr">
+      <c r="B174" s="9" t="inlineStr">
         <is>
           <t>Greet inside 30 seconds. Ask "are you trying to be out by kickoff?" first, then fire accordingly. Card every table before the first round lands. Full hands in, full hands out. Guest issue goes to a manager immediately.</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="32" customHeight="1">
-      <c r="A165" s="8" t="inlineStr">
+    <row r="175" ht="32" customHeight="1">
+      <c r="A175" s="8" t="inlineStr">
         <is>
           <t>HOST</t>
         </is>
       </c>
-      <c r="B165" s="9" t="inlineStr">
+      <c r="B175" s="9" t="inlineStr">
         <is>
           <t>Own the door and own the wait. An accurate quote beats a short one — give a real number, then beat it. First in command runs the book; second in command steps in the moment first gets pulled. Card at the door when the room is young. Keep the line off the sidewalk and feed the wait to the bar.</t>
         </is>
       </c>
     </row>
-    <row r="166" ht="32" customHeight="1">
-      <c r="A166" s="8" t="inlineStr">
+    <row r="176" ht="32" customHeight="1">
+      <c r="A176" s="8" t="inlineStr">
         <is>
           <t>KITCHEN</t>
         </is>
       </c>
-      <c r="B166" s="9" t="inlineStr">
+      <c r="B176" s="9" t="inlineStr">
         <is>
           <t>Prep to game-day pars, confirmed before service. 86 goes to the manager when you see it coming, not when you hit zero. Ticket times called every window. Original position, original condition at every changeover.</t>
         </is>
       </c>
     </row>
-    <row r="167" ht="32" customHeight="1">
-      <c r="A167" s="8" t="inlineStr">
+    <row r="177" ht="32" customHeight="1">
+      <c r="A177" s="8" t="inlineStr">
         <is>
           <t>SOCIAL</t>
         </is>
       </c>
-      <c r="B167" s="9" t="inlineStr">
+      <c r="B177" s="9" t="inlineStr">
         <is>
           <t>Work the room all night, not just the first hour. Get the staff lined up behind the bar during the anthem, buckets landing on tables, the bottle service pour, and the bar at full tilt. Shoot people who want to be shot — ask first, and never a minor, a check, or a POS screen. Post in the game window, not in the crush.</t>
         </is>
       </c>
     </row>
-    <row r="168" ht="32" customHeight="1">
-      <c r="A168" s="8" t="inlineStr">
+    <row r="178" ht="32" customHeight="1">
+      <c r="A178" s="8" t="inlineStr">
         <is>
           <t>SUPPORT</t>
         </is>
       </c>
-      <c r="B168" s="9" t="inlineStr">
+      <c r="B178" s="9" t="inlineStr">
         <is>
           <t>You set the pace of the building. Tables turning is the only thing standing between us and a two-hour wait. Everybody runs food.</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="18" customHeight="1">
-      <c r="A170" s="6" t="inlineStr">
+    <row r="180" ht="18" customHeight="1">
+      <c r="A180" s="6" t="inlineStr">
         <is>
           <t>POST-GAME &amp; CLOSE</t>
         </is>
       </c>
-      <c r="B170" s="7" t="n"/>
-      <c r="C170" s="7" t="n"/>
-      <c r="D170" s="7" t="n"/>
-      <c r="E170" s="7" t="n"/>
-      <c r="F170" s="7" t="n"/>
-      <c r="G170" s="7" t="n"/>
-    </row>
-    <row r="171" ht="17" customHeight="1">
-      <c r="A171" s="24" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B171" s="9" t="inlineStr">
+      <c r="B180" s="7" t="n"/>
+      <c r="C180" s="7" t="n"/>
+      <c r="D180" s="7" t="n"/>
+      <c r="E180" s="7" t="n"/>
+      <c r="F180" s="7" t="n"/>
+      <c r="G180" s="7" t="n"/>
+    </row>
+    <row r="181" ht="17" customHeight="1">
+      <c r="A181" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
         <is>
           <t>All hands on the floor BEFORE the final whistle — not after.</t>
         </is>
       </c>
     </row>
-    <row r="172" ht="17" customHeight="1">
-      <c r="A172" s="24" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B172" s="9" t="inlineStr">
+    <row r="182" ht="17" customHeight="1">
+      <c r="A182" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B182" s="9" t="inlineStr">
         <is>
           <t>Full bottle count and bar inventory tonight, not tomorrow.</t>
         </is>
       </c>
     </row>
-    <row r="173" ht="17" customHeight="1">
-      <c r="A173" s="24" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B173" s="9" t="inlineStr">
+    <row r="183" ht="17" customHeight="1">
+      <c r="A183" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B183" s="9" t="inlineStr">
         <is>
           <t>Every void, comp and discount reconciled to a manager name.</t>
         </is>
       </c>
     </row>
-    <row r="174" ht="17" customHeight="1">
-      <c r="A174" s="24" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B174" s="9" t="inlineStr">
+    <row r="184" ht="17" customHeight="1">
+      <c r="A184" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B184" s="9" t="inlineStr">
         <is>
           <t>Every refusal or cut-off logged with what happened and who made the call.</t>
         </is>
       </c>
     </row>
-    <row r="175" ht="17" customHeight="1">
-      <c r="A175" s="24" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B175" s="9" t="inlineStr">
+    <row r="185" ht="17" customHeight="1">
+      <c r="A185" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B185" s="9" t="inlineStr">
         <is>
           <t>Every station back to original position, original condition.</t>
         </is>
       </c>
     </row>
-    <row r="176" ht="17" customHeight="1">
-      <c r="A176" s="24" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="B176" s="9" t="inlineStr">
+    <row r="186" ht="17" customHeight="1">
+      <c r="A186" s="24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="B186" s="9" t="inlineStr">
         <is>
           <t>Shift notes written: what we ran out of, where the wait broke down, what changes next game.</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="4" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="4" t="inlineStr">
         <is>
           <t>MARKETING:</t>
         </is>
       </c>
     </row>
-    <row r="179" ht="18" customHeight="1">
-      <c r="A179" s="16" t="n"/>
-      <c r="B179" s="17" t="n"/>
-      <c r="C179" s="17" t="n"/>
-      <c r="D179" s="17" t="n"/>
-      <c r="E179" s="17" t="n"/>
-      <c r="F179" s="17" t="n"/>
-      <c r="G179" s="17" t="n"/>
-    </row>
-    <row r="180" ht="18" customHeight="1">
-      <c r="A180" s="17" t="n"/>
-      <c r="B180" s="17" t="n"/>
-      <c r="C180" s="17" t="n"/>
-      <c r="D180" s="17" t="n"/>
-      <c r="E180" s="17" t="n"/>
-      <c r="F180" s="17" t="n"/>
-      <c r="G180" s="17" t="n"/>
-    </row>
-    <row r="182" ht="28" customHeight="1">
-      <c r="A182" s="26" t="inlineStr">
+    <row r="189" ht="18" customHeight="1">
+      <c r="A189" s="16" t="n"/>
+      <c r="B189" s="17" t="n"/>
+      <c r="C189" s="17" t="n"/>
+      <c r="D189" s="17" t="n"/>
+      <c r="E189" s="17" t="n"/>
+      <c r="F189" s="17" t="n"/>
+      <c r="G189" s="17" t="n"/>
+    </row>
+    <row r="190" ht="18" customHeight="1">
+      <c r="A190" s="17" t="n"/>
+      <c r="B190" s="17" t="n"/>
+      <c r="C190" s="17" t="n"/>
+      <c r="D190" s="17" t="n"/>
+      <c r="E190" s="17" t="n"/>
+      <c r="F190" s="17" t="n"/>
+      <c r="G190" s="17" t="n"/>
+    </row>
+    <row r="192" ht="28" customHeight="1">
+      <c r="A192" s="26" t="inlineStr">
         <is>
           <t>100% of our standards, 100% of the time, at 100% volume. A full house is not an excuse to run at 80% — it is the reason we hold the line.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="73">
+  <mergeCells count="82">
+    <mergeCell ref="B145:G145"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="B181:G181"/>
+    <mergeCell ref="B175:G175"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="B147:G147"/>
+    <mergeCell ref="B162:G162"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A117:G117"/>
+    <mergeCell ref="B146:G146"/>
+    <mergeCell ref="A47:G48"/>
+    <mergeCell ref="B173:G173"/>
+    <mergeCell ref="B165:G165"/>
+    <mergeCell ref="B150:G150"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A192:G192"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="B152:G152"/>
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A180:G180"/>
+    <mergeCell ref="B182:G182"/>
+    <mergeCell ref="D51:G51"/>
+    <mergeCell ref="B178:G178"/>
+    <mergeCell ref="A189:G190"/>
+    <mergeCell ref="B183:G183"/>
+    <mergeCell ref="B177:G177"/>
+    <mergeCell ref="B164:G164"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B154:G154"/>
+    <mergeCell ref="B163:G163"/>
+    <mergeCell ref="A35:G36"/>
+    <mergeCell ref="B156:G156"/>
+    <mergeCell ref="D53:G53"/>
+    <mergeCell ref="B155:G155"/>
+    <mergeCell ref="B149:G149"/>
+    <mergeCell ref="D168:G168"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A97:G97"/>
+    <mergeCell ref="B151:G151"/>
+    <mergeCell ref="A96:G96"/>
+    <mergeCell ref="B166:G166"/>
+    <mergeCell ref="A170:G170"/>
+    <mergeCell ref="D169:G169"/>
+    <mergeCell ref="B174:G174"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="B142:G142"/>
+    <mergeCell ref="B160:G160"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="D52:G52"/>
+    <mergeCell ref="A172:G172"/>
+    <mergeCell ref="B144:G144"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="B153:G153"/>
+    <mergeCell ref="B185:G185"/>
+    <mergeCell ref="A169:C169"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A158:G158"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A39:G40"/>
+    <mergeCell ref="B184:G184"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A141:G141"/>
-    <mergeCell ref="A97:G97"/>
-    <mergeCell ref="B145:G145"/>
-    <mergeCell ref="B151:G151"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A96:G96"/>
     <mergeCell ref="B148:G148"/>
-    <mergeCell ref="A158:C158"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="B166:G166"/>
-    <mergeCell ref="B175:G175"/>
-    <mergeCell ref="B171:G171"/>
-    <mergeCell ref="D51:G51"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="B147:G147"/>
-    <mergeCell ref="A170:G170"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A117:G117"/>
     <mergeCell ref="A13:G13"/>
-    <mergeCell ref="B172:G172"/>
-    <mergeCell ref="B174:G174"/>
-    <mergeCell ref="B168:G168"/>
     <mergeCell ref="A31:G31"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="B146:G146"/>
-    <mergeCell ref="A159:C159"/>
+    <mergeCell ref="B186:G186"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="B143:G143"/>
-    <mergeCell ref="A179:G180"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="A182:G182"/>
-    <mergeCell ref="D159:G159"/>
-    <mergeCell ref="B142:G142"/>
-    <mergeCell ref="B164:G164"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="D158:G158"/>
-    <mergeCell ref="A162:G162"/>
-    <mergeCell ref="B154:G154"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="D52:G52"/>
-    <mergeCell ref="A47:G48"/>
-    <mergeCell ref="B163:G163"/>
-    <mergeCell ref="B144:G144"/>
-    <mergeCell ref="B173:G173"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="B153:G153"/>
-    <mergeCell ref="A160:G160"/>
-    <mergeCell ref="B165:G165"/>
-    <mergeCell ref="A35:G36"/>
-    <mergeCell ref="B156:G156"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="B159:G159"/>
+    <mergeCell ref="A56:G56"/>
     <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="D53:G53"/>
-    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A43:G44"/>
-    <mergeCell ref="B150:G150"/>
-    <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A39:G40"/>
-    <mergeCell ref="B155:G155"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="B149:G149"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B167:G167"/>
+    <mergeCell ref="A168:C168"/>
     <mergeCell ref="A76:G76"/>
+    <mergeCell ref="B161:G161"/>
     <mergeCell ref="B176:G176"/>
-    <mergeCell ref="B152:G152"/>
     <mergeCell ref="A138:G139"/>
-    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>